<commit_message>
vault backup: 2026-08-01 21:55:19
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
@@ -1,15 +1,416 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Cards" sheetId="1" r:id="rId1"/>
-    <sheet name="Import Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="Cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Import Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -51,7 +452,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -73,7 +474,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary technology</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -95,7 +496,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary AI</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -117,7 +518,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -139,7 +540,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -161,7 +562,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -183,7 +584,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -205,7 +606,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary AI</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -227,7 +628,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary AI</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -249,7 +650,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -271,7 +672,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -293,7 +694,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary AI</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -315,7 +716,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -337,7 +738,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -359,7 +760,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -381,7 +782,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -403,7 +804,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase technology</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -425,7 +826,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -447,7 +848,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -469,7 +870,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -491,7 +892,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -513,7 +914,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -535,7 +936,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels phrase writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -557,7 +958,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels vocabulary writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -579,7 +980,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels grammar writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -601,7 +1002,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels grammar writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
@@ -623,16 +1024,23 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>外刊精读 Rules_for_supermodels macro writing</t>
+          <t>外刊精读</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -731,5 +1139,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-08-01 23:27:05
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
@@ -36,17 +36,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>calamity</t>
+          <t>come out of disasters/crises</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：大灾难，严重灾祸。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式、严重，比 disaster 更书面，比 accident 更灾难化。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：可指社会、制度、技术或道德层面的重大失败。</t>
+          <t>字面含义：从灾难中产生/走出来
+考研核心考点：灾难后的制度或经验产物
+词汇拆解：come out of = emerge from/result from；disasters = crises/calamities
+熟词辟义/一词多义：come out of 不只是“出来”，还可表示“由……产生”。
+语气色彩：中性偏正式，常用于历史经验、制度改革。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI has not yet caused a calamity, but it might. 作者用 calamity 把 AI 风险提升到公共灾难级别，为“提前监管”铺垫。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：不是普通风险，而是可能触发制度性回应的大危机。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：A powerful technology may bring convenience, but without rules it can also lead to calamity.&lt;br&gt;&lt;b&gt;例句2 社会&lt;/b&gt;：The spread of misinformation could become a public calamity if citizens lose trust in facts.&lt;br&gt;&lt;b&gt;例句3 环境&lt;/b&gt;：Climate change is not a distant inconvenience, but a potential calamity for vulnerable communities.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技伦理、环境保护、公共安全、社会责任。</t>
+          <t>文章语境：文章用它说明很多规则并非预先设计，而是在危机之后被迫形成。
+暗示意思/政治意味/诙谐意味：暗示监管往往滞后：先出事，再补规则。
+特殊考查方式：主旨/推理题会考“某制度为何出现”。
+答题技巧：看到 come out of + 抽象/负面事件，优先译成“源于/产生于”。
+同义替换/错误选项信号：emerge from; result from; be born of; grow out of
+多场景例句：come out of painful lessons；come out of a public-health crisis；come out of market failures
+其他可用地方：社会责任、科技治理、公共安全。
+归一化合并：本卡覆盖这些变体：come out of disasters</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -58,17 +69,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>come out of disasters</t>
+          <t>avert a calamity</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：从灾难中产生。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：制度、规则、改革往往由失败或危机倒逼出来。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：带有历史总结意味，适合议论文开头。</t>
+          <t>字面含义：大灾难；严重灾祸
+考研核心考点：比 disaster 更书面、更严重的负面名词
+词汇拆解：calam- 无需死背；常搭配 natural/political/economic calamity
+熟词辟义/一词多义：可指具体灾害，也可指抽象灾难性后果。
+语气色彩：正式、强负面。</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：New rules often come out of disasters. 作者用美联储、FDA、SEC 的历史证明监管常在灾后出现。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：AI 最好不要等灾难发生后才立规矩。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Better school rules often come out of painful lessons, but wise educators should act earlier.&lt;br&gt;&lt;b&gt;例句2 公共治理&lt;/b&gt;：Many safety standards come out of disasters that reveal hidden weaknesses.&lt;br&gt;&lt;b&gt;例句3 写作模板&lt;/b&gt;：A mature society should not wait for rules to come out of disasters.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：社会责任、科技监管、校园安全、环境治理。</t>
+          <t>文章语境：文章用它指 AI 失控或监管失败可能造成的大灾难。
+暗示意思/政治意味/诙谐意味：带有警告色彩，让风险显得不是小故障而是系统性灾难。
+特殊考查方式：态度题中常指作者担忧或警惕。
+答题技巧：遇到 calamity 不要译轻，选项里 catastrophe/crisis 常是替换。
+同义替换/错误选项信号：catastrophe; disaster; crisis; debacle
+多场景例句：avert a calamity；a financial calamity；a public calamity caused by negligence
+其他可用地方：环境灾害、公共安全、科技风险。
+归一化合并：本卡覆盖这些变体：calamity</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -85,12 +107,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：自愿性标准，非强制规范。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：行业自律、软性监管。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：中性，但在公共风险语境中可能暗示“不够硬”。</t>
+          <t>字面含义：自愿性标准
+考研核心考点：政策类阅读常见：非强制监管工具
+词汇拆解：voluntary = 自愿的；standards = standards/rules/benchmarks
+熟词辟义/一词多义：standard 不只是“标准答案”，还指行业规范。
+语气色彩：正式、中性，但常暗示约束力不足。</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：政府与 AI 公司制定 voluntary standards，但作者认为现有努力混乱。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：只靠企业自愿可能不够，需要制度化 formalise。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：Voluntary standards can guide innovation, but they cannot replace public accountability.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：Companies may adopt voluntary standards to protect employee data.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：When public safety is at stake, voluntary standards should be backed by clear rules.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI 监管、企业社会责任、食品安全、平台治理。</t>
+          <t>文章语境：文章讨论 AI 公司是否只靠自愿标准就足够。
+暗示意思/政治意味/诙谐意味：暗示企业自律可能不可靠，需要公共监管。
+特殊考查方式：细节题会问措施性质：mandatory 还是 voluntary。
+答题技巧：看到 voluntary standards，要留意作者是否认为其 too weak。
+同义替换/错误选项信号：self-imposed rules; non-binding guidelines; industry standards
+多场景例句：adopt voluntary standards；rely on voluntary safety standards；turn voluntary standards into binding rules
+其他可用地方：科技监管、企业责任、行业自律。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -102,17 +134,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>guardrailed</t>
+          <t>a guardrailed release / guardrail a model</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：加了护栏/安全限制的。&lt;br&gt;&lt;b&gt;AI 语境&lt;/b&gt;：指模型被设置安全边界，不能随意回答危险请求。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：被制度、规则或技术限制住。</t>
+          <t>字面含义：被护栏限制的；设有安全边界的
+考研核心考点：科技语境中的新用法：给系统加安全限制
+词汇拆解：guardrail = 护栏/防护栏；-ed 表示“被设置防护”。
+熟词辟义/一词多义：guardrail 从道路护栏引申为政策/技术边界。
+语气色彩：技术政策语体，中性偏谨慎。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Fable 是 Mythos 的 guardrailed version。作者暗示即使“加了护栏”，政府仍然不放心。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：护栏不等于绝对安全，也可能成为政治争论的焦点。&lt;br&gt;&lt;b&gt;例句1 AI&lt;/b&gt;：A guardrailed model may refuse harmful instructions, but its underlying capability remains powerful.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Children need guardrailed access to the internet rather than total isolation from technology.&lt;br&gt;&lt;b&gt;例句3 管理&lt;/b&gt;：Innovation should be encouraged, but guardrailed by ethical principles.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI 安全、青少年上网、科技伦理、教育技术。</t>
+          <t>文章语境：文章用它形容受安全规则限制的 AI 模型。
+暗示意思/政治意味/诙谐意味：暗示模型能力很强，需要边界防止滥用。
+特殊考查方式：词义题可能考从具体护栏到抽象安全边界。
+答题技巧：译成“设有安全护栏/受安全限制”，不要死译成“有栏杆的”。
+同义替换/错误选项信号：safeguarded; constrained; safety-bounded
+多场景例句：guardrailed AI systems；a guardrailed release；guardrails against misuse
+其他可用地方：科技生活、AI 安全、制度设计。
+归一化合并：本卡覆盖这些变体：guardrailed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -124,17 +167,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>slap sb/sth with controls</t>
+          <t>export controls</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：突然对某人/某物施加管制或处罚。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻英语，动作感强，常暗示粗暴、突然、行政性强。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：be slapped with sanctions / fines / export controls。</t>
+          <t>字面含义：出口管制
+考研核心考点：国际关系/科技竞争高频政策词
+词汇拆解：export = 出口；controls = 管制措施
+熟词辟义/一词多义：control 在政策语境中多译为“管制/限制”。
+语气色彩：正式、政治经济色彩强。</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Anthropic was slapped with export controls. 作者用 slapped 表示政府动作突然且带惩罚色彩。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：不是温和监管，而是行政力量直接压下去。&lt;br&gt;&lt;b&gt;例句1 国际关系&lt;/b&gt;：The company was slapped with sanctions after violating export rules.&lt;br&gt;&lt;b&gt;例句2 社会&lt;/b&gt;：Platforms that ignore child safety may be slapped with heavy fines.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Punishment alone is not enough; firms also need clear guidance before they are slapped with penalties.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：法律监管、国际制裁、平台治理、企业责任。</t>
+          <t>文章语境：文章涉及美国限制高端 AI 芯片或模型流向中国。
+暗示意思/政治意味/诙谐意味：暗示国家安全与自由贸易之间的冲突。
+特殊考查方式：细节题会用 restrictions/curbs 替换 controls。
+答题技巧：遇到 export controls，定位政府干预与战略利益。
+同义替换/错误选项信号：export restrictions; trade curbs; technology controls
+多场景例句：tighten export controls；be subject to export controls；export controls on advanced chips
+其他可用地方：科技竞争、国际贸易、国家安全。</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -151,12 +204,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：边做边定规则，临时拼凑规则。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：批评性强，暗示不专业、不稳定、缺少制度设计。&lt;br&gt;&lt;b&gt;熟词&lt;/b&gt;：on the fly = 临时地、现场地、边进行边处理。</t>
+          <t>字面含义：临时编规则；边做边定规则
+考研核心考点：熟词短语：on the fly = 即时地、临场地
+词汇拆解：make up = 编造/制定；rules = 规则；on the fly = without prior planning
+熟词辟义/一词多义：make up 不只是“化妆/组成”，可指“编造、临时凑出”。
+语气色彩：口语化、批评性，暗示缺乏制度性。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：政府似乎在 make up rules on the fly。作者批评其 AI 监管没有清晰原则。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：政策不是 rule-based，而是 improvisation。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Schools should not make up rules on the fly when dealing with AI homework.&lt;br&gt;&lt;b&gt;例句2 政策&lt;/b&gt;：A government that makes up rules on the fly will lose public trust.&lt;br&gt;&lt;b&gt;例句3 职场&lt;/b&gt;：Managers should not make up rules on the fly whenever a problem appears.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：公共治理、学校管理、职场制度、AI 监管。</t>
+          <t>文章语境：文章批评政府对 AI 的规则可能是临时应付。
+暗示意思/政治意味/诙谐意味：暗示监管混乱、反应式治理，而非成熟制度。
+特殊考查方式：态度题中是负面信号。
+答题技巧：看到 on the fly，理解为“临时/即时”，不是“在飞行中”。
+同义替换/错误选项信号：improvise rules; ad-lib regulations; set rules case by case
+多场景例句：make up policy on the fly；make up safety rules on the fly；govern a new industry on the fly
+其他可用地方：科技治理、公共管理、制度建设。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -173,12 +236,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：民族主义色彩。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：tinge 本义是淡淡的颜色，引申为某种意味、倾向、色彩。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：通常带轻微负面，表示某种立场不完全明说但能感觉到。</t>
+          <t>字面含义：民族主义色彩；国家主义意味
+考研核心考点：态度与立场词：tinge 表示淡淡的色彩/倾向
+词汇拆解：nationalistic = 民族主义的；tinge = slight trace/color
+熟词辟义/一词多义：tinge 可指颜色，也可指情绪、政治色彩。
+语气色彩：含蓄批评，journalistic。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 政策带有 unpleasant nationalistic tinge。作者批评美国优先主义。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：不是纯粹安全监管，而混入“美国人优先”的意识形态。&lt;br&gt;&lt;b&gt;例句1 国际关系&lt;/b&gt;：The policy has a nationalistic tinge, even though it is presented as a security measure.&lt;br&gt;&lt;b&gt;例句2 文化&lt;/b&gt;：Patriotism can inspire responsibility, but a nationalistic tinge may narrow people's worldview.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Global challenges require cooperation, not policies with a narrow nationalistic tinge.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：国际合作、文化交流、科技竞争、全球治理。</t>
+          <t>文章语境：文章说某些 AI 政策带有国家主义色彩。
+暗示意思/政治意味/诙谐意味：暗示政策不只是安全考虑，也有国家竞争和情绪动员。
+特殊考查方式：推理题可能问作者如何看待政策动机。
+答题技巧：不要译成“民族颜色”，应译为“民族主义意味”。
+同义替换/错误选项信号：nationalist flavour; patriotic colouring; political undertone
+多场景例句：a nationalistic tinge in trade policy；a nationalistic tinge to the debate；policy with a nationalist undertone
+其他可用地方：国际关系、科技竞争、政治态度。</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -195,12 +268,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：优先于，重要性高于。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式、议论文高频，用于排序价值和原则。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：safety / public interest / education / long-term development takes precedence over profit / convenience。</t>
+          <t>字面含义：优先于；凌驾于
+考研核心考点：写作高分逻辑短语：表达价值排序
+词汇拆解：precedence = priority；take precedence over A = be more important than A
+熟词辟义/一词多义：precedence 与 precedent 不同：前者优先权，后者先例。
+语气色彩：正式、中性。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Americans' AI access takes precedence over foreigners'. 作者指出美国政府把本国访问权放在外国人之前。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：表面是安全监管，实际涉及利益排序。&lt;br&gt;&lt;b&gt;例句1 作文&lt;/b&gt;：Public safety should take precedence over commercial profit.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：In education, students' long-term growth should take precedence over short-term scores.&lt;br&gt;&lt;b&gt;例句3 环境&lt;/b&gt;：Environmental protection must take precedence over reckless expansion.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：社会责任、教育、环境、科技伦理、公共利益。</t>
+          <t>文章语境：文章讨论安全、主权或战略利益是否优先于市场开放。
+暗示意思/政治意味/诙谐意味：暗示价值冲突：安全 vs 创新/开放/商业利益。
+特殊考查方式：翻译题常考抽象名词的主谓搭配。
+答题技巧：选项里 priority/come before 常是同义替换。
+同义替换/错误选项信号：come before; outweigh; be given priority over
+多场景例句：safety takes precedence over speed；public interest takes precedence over private profit；long-term stability takes precedence over short-term gains
+其他可用地方：作文：社会责任、科技伦理、公共利益。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -212,17 +295,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>frontier AI</t>
+          <t>frontier AI models</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：前沿人工智能，能力处于最前沿的 AI 系统。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：代表未知边界、高潜力、高风险。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：技术政策词，常和 regulation, safety, governance 搭配。</t>
+          <t>字面含义：前沿人工智能；最先进 AI
+考研核心考点：科技类核心术语
+词汇拆解：frontier = 边界/前沿；AI = artificial intelligence
+熟词辟义/一词多义：frontier 不只是“边疆”，也指研究或技术最前沿。
+语气色彩：正式、技术政策语体。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Regulating frontier AI is tricky. 作者承认前沿 AI 很难监管。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：frontier 不是普通技术，而是靠近能力边界和风险边界。&lt;br&gt;&lt;b&gt;例句1 AI&lt;/b&gt;：Frontier AI may transform research, but it also requires careful oversight.&lt;br&gt;&lt;b&gt;例句2 经济&lt;/b&gt;：Countries that lead in frontier AI may gain enormous economic leverage.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：When frontier technologies enter daily life, ethical rules must keep pace.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、国家竞争、科技伦理、社会治理。</t>
+          <t>文章语境：文章讨论最强模型的监管和开放问题。
+暗示意思/政治意味/诙谐意味：暗示这些模型能力未知、风险更高、监管更敏感。
+特殊考查方式：细节题会用 cutting-edge/advanced 替换。
+答题技巧：翻译时加“前沿/最先进”，不要译成“边境 AI”。
+同义替换/错误选项信号：advanced AI; cutting-edge AI; state-of-the-art models
+多场景例句：frontier AI models；frontier AI regulation；risks posed by frontier AI
+其他可用地方：科技生活、AI 治理、创新与安全。
+归一化合并：本卡覆盖这些变体：frontier AI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -234,17 +328,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>open-weight</t>
+          <t>open-weight AI models</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：开放权重的，模型参数可被获取、运行或改动。&lt;br&gt;&lt;b&gt;区分&lt;/b&gt;：open-weight 不完全等于 open-source；代码、训练数据、许可证未必完全开放。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：AI 治理关键词。</t>
+          <t>字面含义：开放权重的
+考研核心考点：AI 术语：模型参数可公开获取/下载
+词汇拆解：open = 开放；weight = 模型权重/参数，不是体重。
+熟词辟义/一词多义：weight 在 AI 中指参数；熟词僻义很关键。
+语气色彩：技术语体，中性但政策敏感。</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：中国许多顶尖模型是 open-weight，任何人都能 run or tinker with them。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：开放降低门槛，也让封锁更难执行。&lt;br&gt;&lt;b&gt;例句1 AI&lt;/b&gt;：Open-weight models spread quickly because researchers can adapt them to local needs.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Open tools can reduce inequality if students are taught how to use them responsibly.&lt;br&gt;&lt;b&gt;例句3 政策&lt;/b&gt;：A ban on open-weight models is difficult to enforce once the files are widely available.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：技术开放、知识共享、风险控制、教育公平。</t>
+          <t>文章语境：文章讨论开放权重模型一旦发布就难以收回。
+暗示意思/政治意味/诙谐意味：暗示开放带来创新，也带来失控和滥用风险。
+特殊考查方式：词义题可能考 weight 的技术义。
+答题技巧：看到 open-weight，要想到可复制、可改造、难封禁。
+同义替换/错误选项信号：open-source-like models; publicly available weights
+多场景例句：open-weight AI models；release open weights；risks of open-weight systems
+其他可用地方：科技创新、开放知识、风险治理。
+归一化合并：本卡覆盖这些变体：open-weight</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -256,17 +361,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tinker with</t>
+          <t>tinker/fiddle with safety protections</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：摆弄、修修补补、小幅改动。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：比 modify 口语、更随意，暗示非正式实验。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：也可指对制度或政策做小修小补。</t>
+          <t>字面含义：摆弄/篡改了它的安全保护
+考研核心考点：fiddle with = 胡乱改动，语气比 modify 更轻佻
+词汇拆解：fiddle = 摆弄；safety protections = 安全保护措施
+熟词辟义/一词多义：fiddle with 常暗示不专业或不该改。
+语气色彩：批评、带轻微调侃。</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：anyone can run or tinker with open-weight models。开放权重让使用者不只是使用，还能改造。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：Students learn programming faster when they can tinker with real code.&lt;br&gt;&lt;b&gt;例句2 政策&lt;/b&gt;：The government keeps tinkering with rules instead of redesigning the system.&lt;br&gt;&lt;b&gt;例句3 学习&lt;/b&gt;：Instead of memorising blindly, learners should tinker with sentence patterns and use them in new contexts.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：技术学习、教育方法、制度改革、产品迭代。</t>
+          <t>文章语境：文章指用户或开发者改动模型安全机制。
+暗示意思/政治意味/诙谐意味：暗示安全护栏可能被轻易绕过。
+特殊考查方式：态度题可判断作者担心滥用。
+答题技巧：译为“乱改/摆弄”，不要中性译为“调整”。
+同义替换/错误选项信号：tamper with; tinker with; mess with; alter
+多场景例句：fiddle with safety protections；tamper with warning systems；mess with privacy settings
+其他可用地方：科技安全、个人责任、平台治理。
+归一化合并：本卡覆盖这些变体：tinker with；fiddled with its safety protections；tinker with them</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -278,17 +394,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>crack down on</t>
+          <t>crack down on distillation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：严厉打击，强力整治。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政府/执法语境强，带控制、惩罚意味。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：crack down on illegal trade / data abuse / exam cheating / pollution。</t>
+          <t>字面含义：严厉打击知识蒸馏/能力提炼
+考研核心考点：科技监管 + 熟词僻义组合
+词汇拆解：crack down on = 严打；distillation = AI 知识蒸馏/能力提炼
+熟词辟义/一词多义：distillation 不是化学蒸馏，而是模型能力转移。
+语气色彩：强监管、技术敏感。</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：American labs are cracking down on distillation. 美国实验室打击竞争者用强模型输出训练自己的模型。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：不仅是技术问题，也涉及技术垄断和竞争壁垒。&lt;br&gt;&lt;b&gt;例句1 社会&lt;/b&gt;：Authorities should crack down on companies that misuse personal data.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Schools may crack down on cheating, but they also need to teach academic integrity.&lt;br&gt;&lt;b&gt;例句3 环境&lt;/b&gt;：Governments must crack down on factories that ignore pollution standards.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：法律、教育诚信、环境保护、平台治理。</t>
+          <t>文章语境：文章讨论限制通过蒸馏绕过模型管制。
+暗示意思/政治意味/诙谐意味：暗示开放与封锁之间存在技术绕道。
+特殊考查方式：细节题问政府措施时，该短语是定位点。
+答题技巧：不要死译“打击蒸馏”，要译“整治知识蒸馏/能力转移”。
+同义替换/错误选项信号：clamp down on model distillation; curb capability extraction; restrict knowledge transfer
+多场景例句：cracking down on distillation；curbing model distillation；restricting the extraction of model capabilities
+其他可用地方：AI 安全、知识产权、科技治理。
+归一化合并：本卡覆盖这些变体：crack down on；cracking down on distillation</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -305,12 +432,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：蒸馏。&lt;br&gt;&lt;b&gt;AI 语境&lt;/b&gt;：用强模型的输出训练较小或竞争模型。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：把复杂能力压缩、转移或提炼到另一个系统中。</t>
+          <t>字面含义：蒸馏；提炼；AI 中的知识蒸馏
+考研核心考点：熟词僻义：从化学提纯引申为知识/模型能力提炼
+词汇拆解：distil/distill = 蒸馏、提炼；-ation 名词后缀
+熟词辟义/一词多义：AI 里指用强模型训练弱模型，转移能力。
+语气色彩：技术语体，中性，但政策语境下敏感。</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：美国实验室打击 distillation，因为它可能帮助竞争者追赶。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：知识一旦可通过输出转移，技术优势就更难长期封锁。&lt;br&gt;&lt;b&gt;例句1 AI&lt;/b&gt;：Distillation can make powerful AI capabilities cheaper and easier to deploy.&lt;br&gt;&lt;b&gt;例句2 学习&lt;/b&gt;：Good notes are a form of distillation: they turn complex arguments into usable ideas.&lt;br&gt;&lt;b&gt;例句3 写作&lt;/b&gt;：Education should help students distil information into judgment, not merely collect facts.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI、学习方法、知识管理、教育写作。</t>
+          <t>文章语境：文章指通过 distillation 将受限模型能力转移到开放模型。
+暗示意思/政治意味/诙谐意味：暗示管制可能被技术绕过。
+特殊考查方式：词义题/翻译题会考是否能识别 AI 语境。
+答题技巧：不要译成普通“蒸馏”，应译为“知识蒸馏/能力提炼”。
+同义替换/错误选项信号：knowledge distillation; model distillation; extract capabilities
+多场景例句：model distillation techniques；distillation of a powerful model；crack down on distillation
+其他可用地方：AI 学习、技术扩散、监管漏洞。</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -322,17 +459,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>unworkable</t>
+          <t>an unworkable regulatory scheme</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：行不通的，不可操作的。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政策评估词，强调方案在现实中无法执行。&lt;br&gt;&lt;b&gt;近义&lt;/b&gt;：impractical, infeasible；但 unworkable 更像“机制上跑不通”。</t>
+          <t>字面含义：行不通的；不可操作的
+考研核心考点：政策评价词，强烈负面
+词汇拆解：un- = not；workable = 可行的
+熟词辟义/一词多义：workable 不是“能工作的”，而是“可执行/可操作”。
+语气色彩：正式、批评性。</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：A permanent block is unworkable. 永久封锁 AI 模型不现实。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：作者不是反对监管，而是反对无效监管。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：A total ban on smartphones in education may be unworkable.&lt;br&gt;&lt;b&gt;例句2 环境&lt;/b&gt;：Environmental rules become unworkable if they ignore local economic realities.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：A policy that sounds strict may still be unworkable in practice.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：政策批判、教育改革、技术治理、经济管理。</t>
+          <t>文章语境：文章评价某些监管方案可能难以执行。
+暗示意思/政治意味/诙谐意味：暗示方案理论上好听，现实中落不了地。
+特殊考查方式：态度题中 negative/critical。
+答题技巧：选项 feasible/practical 是反义，impractical 是同义。
+同义替换/错误选项信号：impractical; infeasible; impossible to enforce
+多场景例句：an unworkable ban；an unworkable regulatory scheme；rules that are technically unworkable
+其他可用地方：政策评估、科技治理、作文批判。
+归一化合并：本卡覆盖这些变体：unworkable</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -344,17 +492,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>malleable</t>
+          <t>cheap and malleable AI models</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：可塑的，易调整的。&lt;br&gt;&lt;b&gt;本义&lt;/b&gt;：金属等可锤打成形。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：想法、制度、模型、性格或学习方法容易被塑造。</t>
+          <t>字面含义：便宜且可塑/易改造的
+考研核心考点：双形容词并列，描述技术扩散条件
+词汇拆解：cheap = 成本低；malleable = 易被改变/改造
+熟词辟义/一词多义：cheap 不总是贬义，可指低成本；malleable 可褒可贬。
+语气色彩：中性中带风险。</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Chinese models are cheap and malleable. 便宜且容易改造，所以很有吸引力。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：malleable 不只是“灵活”，还暗示可被不同用户用于不同目的。&lt;br&gt;&lt;b&gt;例句1 AI&lt;/b&gt;：Malleable models are attractive because firms can adapt them to specific tasks.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Young minds are malleable, so good habits should be formed early.&lt;br&gt;&lt;b&gt;例句3 写作&lt;/b&gt;：A malleable learning system can serve students with different needs.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育学习、AI 应用、个人品质、制度设计。</t>
+          <t>文章语境：文章用它说明开放模型为什么容易普及和被改造。
+暗示意思/政治意味/诙谐意味：暗示低成本 + 可改造 = 创新机会与滥用风险并存。
+特殊考查方式：推理题可能问为什么难以控制。
+答题技巧：看到并列形容词，注意共同服务于后面的名词。
+同义替换/错误选项信号：low-cost and adaptable; inexpensive and easy to modify
+多场景例句：cheap and malleable AI models；cheap and adaptable tools；low-cost and easy-to-modify technology
+其他可用地方：科技生活、教育工具、创新风险。
+归一化合并：本卡覆盖这些变体：malleable；cheap and malleable</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -366,17 +525,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>a gulf between A and B</t>
+          <t>a gulf between publicly available and restricted models</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：A 与 B 之间的巨大鸿沟。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：比 gap 更强，常表示难以跨越的差距。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：a gulf between rich and poor / policy and reality / public and restricted models。</t>
+          <t>字面含义：公开可用模型与受限模型之间的巨大差距是个问题
+考研核心考点：抽象主语 + 系表结构
+词汇拆解：publicly available = 公开可得；restricted = 受限制的；gulf = 巨大差距
+熟词辟义/一词多义：available 是“可获得的”，不是“有空的”；restricted 是“受限的”。
+语气色彩：正式、问题判断。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a gulf between publicly available and restricted models。公开模型与受限模型之间能力差太大，会造成社会适应问题。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：不平等访问会制造权力集中。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：There is a gulf between students who can use AI wisely and those who cannot.&lt;br&gt;&lt;b&gt;例句2 社会&lt;/b&gt;：A gulf between urban and rural education can damage equal opportunity.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Technology should narrow, not widen, the gulf between different social groups.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育公平、数字鸿沟、贫富差距、科技伦理。</t>
+          <t>文章语境：文章指出模型能力若分化过大，会使发布时造成冲击。
+暗示意思/政治意味/诙谐意味：暗示过度封锁可能制造技术断层。
+特殊考查方式：翻译题考多重前置修饰和 A-B 对比。
+答题技巧：先抓主干：a gulf is a problem；中间是 between 短语。
+同义替换/错误选项信号：a divide between open and closed systems; a gap between public and restricted access
+多场景例句：a gulf between urban and rural education is a problem；a gulf between rich and poor is a problem；a gap between innovation and regulation is a problem
+其他可用地方：教育公平、科技鸿沟、社会责任。
+归一化合并：本卡覆盖这些变体：a gulf between A and B；a gulf between publicly available and restricted models is a problem.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -388,17 +558,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bottle up</t>
+          <t>bottle up powerful technology</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：封存、压住、不让释放。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：bottle 是瓶子；bottle up 像把东西装进瓶里憋住。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：形象，有压抑后突然爆发的暗示。</t>
+          <t>字面含义：压住；封锁；憋住；限制流动
+考研核心考点：短语动词，常用于情绪、信息、技术扩散
+词汇拆解：bottle = 瓶子；bottle up = 把……装瓶里，引申为压住。
+熟词辟义/一词多义：可指压抑情绪，也可指封锁资源/信息。
+语气色彩：形象、略口语。</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：regulators bottled up several generations of AI advances。监管者如果把几代进步都封起来，最终释放会更混乱。&lt;br&gt;&lt;b&gt;暗示/诙谐&lt;/b&gt;：技术进步像气体或压力，被封住越久越危险。&lt;br&gt;&lt;b&gt;例句1 情绪&lt;/b&gt;：Students should not bottle up stress before exams.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：Bottling up innovation may create a sudden and disruptive release later.&lt;br&gt;&lt;b&gt;例句3 社会&lt;/b&gt;：Public anger was bottled up for years before it finally erupted.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技治理、心理健康、社会矛盾、教育压力。</t>
+          <t>文章语境：文章用它描述把强模型能力长期封住不放。
+暗示意思/政治意味/诙谐意味：暗示被压住的力量最终可能突然爆发。
+特殊考查方式：词义题会考非字面义。
+答题技巧：对象若是 emotion/information/technology，译为“压抑/封锁/限制”。
+同义替换/错误选项信号：hold back; contain; suppress; lock up
+多场景例句：bottle up public anger；bottle up innovation；bottle up powerful technology
+其他可用地方：科技扩散、心理健康、社会治理。
+归一化合并：本卡覆盖这些变体：bottle up</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -415,12 +596,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：分阶段发布、错峰发布。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：把风险分散，让社会逐步适应。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政策设计词，强调节奏控制。</t>
+          <t>字面含义：分阶段发布；错峰释放
+考研核心考点：科技产品/政策执行类实用搭配
+词汇拆解：staggered = 分阶段的/错开的；release = 发布/释放
+熟词辟义/一词多义：release 不只是“释放犯人”，也指产品发布、模型开放。
+语气色彩：正式、中性。</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：an evaluation period and a staggered release to trusted institutions。先评估，再分阶段给可信机构使用。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：作者支持释放模型，但要控制节奏和对象。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：A staggered release can reduce the shock of powerful new technologies.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Schools can introduce AI tools through a staggered release rather than a sudden rollout.&lt;br&gt;&lt;b&gt;例句3 公共政策&lt;/b&gt;：Major reforms often work better with staggered implementation.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI 发布、教育改革、公共政策、产品上线。</t>
+          <t>文章语境：文章提出分阶段释放模型以避免能力突然跃升。
+暗示意思/政治意味/诙谐意味：暗示渐进管理比一次性开放更稳。
+特殊考查方式：细节题会把 staggered 替换为 phased/gradual。
+答题技巧：翻译为“分阶段发布”，不要译成“蹒跚发布”。
+同义替换/错误选项信号：phased release; gradual rollout; controlled release
+多场景例句：a staggered release of AI models；a phased release schedule；gradual rollout of new rules
+其他可用地方：科技治理、产品发布、政策改革。</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -432,17 +623,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>formalise</t>
+          <t>formalise safety rules</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：使正式化，使制度化。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：把临时做法、默契或自愿规范变成明确规则。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，常用于制度建设。</t>
+          <t>字面含义：使正式化；把……制度化
+考研核心考点：制度建设高频动词
+词汇拆解：formal = 正式的；-ise = 使……化
+熟词辟义/一词多义：不是“形式化”那么空，可译为“确立正式制度”。
+语气色彩：正式、中性偏政策。</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：分阶段发布是 good start, but it needs formalising。作者认为惯例还不够，要形成制度。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：临时协商不可靠，制度化才可持续。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：AI safety practices should be formalised before models become widely available.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：Flexible work can succeed if expectations are formalised.&lt;br&gt;&lt;b&gt;例句3 教育&lt;/b&gt;：Schools should formalise rules for the responsible use of AI tools.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：制度建设、职场管理、教育规范、科技治理。</t>
+          <t>文章语境：文章建议把临时规则正式化。
+暗示意思/政治意味/诙谐意味：暗示从临时应对走向制度化治理。
+特殊考查方式：写作中可用于制度、标准、程序。
+答题技巧：看到 formalise + arrangement/rules/process，译为“将……制度化”。
+同义替换/错误选项信号：institutionalise; codify; make official
+多场景例句：formalise safety standards；formalise informal rules；formalise cooperation between schools and firms
+其他可用地方：制度建设、职场流程、科技监管。
+归一化合并：本卡覆盖这些变体：formalise；formalising</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -459,12 +661,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：微观管理，过度干预细节。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：明显负面，表示领导者不懂放权。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：政治人物不应干预技术评估细节。</t>
+          <t>字面含义：事无巨细地管理；过度干预
+考研核心考点：管理类负面词
+词汇拆解：micro = 微小；manage = 管理
+熟词辟义/一词多义：不是普通 manage，而是管得过细。
+语气色彩：批评性。</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：politicians should not be micromanaging the process。作者区分政治目标与技术执行。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：民主领导人定目标，专家做评估。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Parents should guide children, but not micromanage every minute of their study.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：A good manager sets goals instead of micromanaging every task.&lt;br&gt;&lt;b&gt;例句3 政策&lt;/b&gt;：Governments should regulate platforms, but they should not micromanage technical design.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：职场、教育、公共治理、科技监管。</t>
+          <t>文章语境：文章警惕政府不要逐项管死 AI 公司技术细节。
+暗示意思/政治意味/诙谐意味：暗示监管需要边界，避免抑制创新。
+特殊考查方式：态度题负面；常与 bureaucracy 搭配。
+答题技巧：译为“过度干预/微观管理”，不要只译“管理”。
+同义替换/错误选项信号：overmanage; interfere in details; regulate every detail
+多场景例句：micromanage AI companies；micromanage classroom teaching；micromanage employees' daily work
+其他可用地方：职场管理、教育管理、政府监管。</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -476,17 +688,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>horse-trade</t>
+          <t>horse-trade with AI companies</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：讨价还价，政治交易。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：贬义，暗示原则被交易替代。&lt;br&gt;&lt;b&gt;诙谐/讽刺&lt;/b&gt;：原指买马卖马时讨价还价，转用于政治或商业交易，带粗俗现实感。</t>
+          <t>字面含义：与 AI 公司讨价还价/利益交换
+考研核心考点：具体化的政治经济搭配
+词汇拆解：horse-trading = 幕后交易/讨价还价；with AI companies = 对象
+熟词辟义/一词多义：horse-trading 比 negotiation 更带利益交换味。
+语气色彩：新闻批评语气。</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：politicians should not be horse-trading with AI companies。作者批评当前监管像政治交易。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：技术安全不应被公司利益和政治权力私下交换。&lt;br&gt;&lt;b&gt;例句1 政治&lt;/b&gt;：Public health should not be reduced to horse-trading between politicians and companies.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Education policy needs principles, not horse-trading among interest groups.&lt;br&gt;&lt;b&gt;例句3 社会责任&lt;/b&gt;：When safety is at stake, horse-trading can undermine public trust.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：政治批评、商业伦理、社会责任、公共安全。</t>
+          <t>文章语境：文章警惕政府规则被与大公司谈判塑形。
+暗示意思/政治意味/诙谐意味：暗示大公司可能凭资源影响公共规则。
+特殊考查方式：推理题可考 regulatory capture。
+答题技巧：译出“讨价还价/利益交换”，不要中性化成“合作”。
+同义替换/错误选项信号：bargaining with firms; cutting deals with companies; regulatory horse-trading
+多场景例句：horse-trading with AI companies；horse-trading with industry giants；behind-the-scenes bargaining with platforms
+其他可用地方：企业责任、科技监管、公共伦理。
+归一化合并：本卡覆盖这些变体：horse-trade；horse-trading with AI companies</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -503,12 +726,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：退后一步，不插手细节。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：在设定目标后给专家、市场或执行者空间。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：理性克制，常用于治理分工。</t>
+          <t>字面含义：退后观察；暂不干预
+考研核心考点：熟词短语：stand 不只是站立
+词汇拆解：stand back = move away / refrain from intervening
+熟词辟义/一词多义：可指身体退后，也可指政策上不插手。
+语气色彩：中性，政策语境中可能暗示克制。</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Once those goals are set, politicians should stand back. 政治人物设定风险目标后应让技术评估者工作。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：好治理不是缺席，而是边界清晰。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Once learning goals are clear, teachers should stand back and let students explore.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：Leaders should stand back after giving teams a clear direction.&lt;br&gt;&lt;b&gt;例句3 政策&lt;/b&gt;：Politicians should stand back when scientific expertise is required.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育、职场领导、科技治理、专家决策。</t>
+          <t>文章语境：文章说监管者有时应退一步看整体。
+暗示意思/政治意味/诙谐意味：暗示不要过度干预，要保留创新空间。
+特殊考查方式：词义题常考抽象义“旁观/不插手”。
+答题技巧：结合对象判断：stand back from markets = 不干预市场。
+同义替换/错误选项信号：step back; refrain from intervening; take a broader view
+多场景例句：stand back from daily management；stand back and assess the risks；stand back from micromanaging firms
+其他可用地方：职场管理、政策监管、个人决策。</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -520,17 +753,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>amalgamate</t>
+          <t>amalgamate rules/agencies</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：整合、合并。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，常用于把不同来源的信息、机构、资源合并。&lt;br&gt;&lt;b&gt;区别&lt;/b&gt;：比 combine 更书面，强调融合成一个整体。</t>
+          <t>字面含义：合并；整合
+考研核心考点：正式动词，常用于机构、规则、系统
+词汇拆解：amalgam = 混合物；-ate 动词化
+熟词辟义/一词多义：比 combine 更正式，强调合成一个整体。
+语气色彩：正式、中性。</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：amalgamate knowledge from AI labs, research groups and foreign bodies。AI 监管需要整合多方专业知识。&lt;br&gt;&lt;b&gt;例句1 学习&lt;/b&gt;：Good writing amalgamates evidence, logic and personal judgment.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：AI governance should amalgamate expertise from engineers, lawyers and ethicists.&lt;br&gt;&lt;b&gt;例句3 职场&lt;/b&gt;：A strong team can amalgamate different skills into one practical solution.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：知识整合、团队合作、科技治理、作文表达升级。</t>
+          <t>文章语境：文章建议把分散的 AI 监管资源或规则整合起来。
+暗示意思/政治意味/诙谐意味：暗示碎片化监管需要统一协调。
+特殊考查方式：阅读中常与 agencies/data/rules 搭配。
+答题技巧：选项 merge/integrate/consolidate 是同义替换。
+同义替换/错误选项信号：merge; integrate; consolidate; combine
+多场景例句：amalgamate regulatory agencies；amalgamate scattered rules；amalgamate data from different sources
+其他可用地方：制度建设、组织管理、科技治理。
+归一化合并：本卡覆盖这些变体：amalgamate</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -542,17 +786,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>build leverage</t>
+          <t>build leverage over AI companies</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：建立筹码，增强议价能力。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：leverage 本义为杠杆，引申为影响力、筹码、可支配优势。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：战略性强，常用于国家、企业、个人竞争。</t>
+          <t>字面含义：建立筹码；增强谈判/影响力
+考研核心考点：政治经济类核心搭配
+词汇拆解：leverage = 杠杆；引申为影响力/谈判筹码
+熟词辟义/一词多义：leverage 不是普通“杠杆”，常指可利用的权力优势。
+语气色彩：正式、策略色彩。</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Other countries must build leverage with their own AI sectors and regulations. 其他国家不能完全被美国出口管制牵着走。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：技术自主就是谈判筹码。&lt;br&gt;&lt;b&gt;例句1 个人发展&lt;/b&gt;：Young people can build leverage by mastering skills that are hard to replace.&lt;br&gt;&lt;b&gt;例句2 国家竞争&lt;/b&gt;：Countries build leverage when they develop independent technologies.&lt;br&gt;&lt;b&gt;例句3 职场&lt;/b&gt;：A worker with rare expertise has more leverage in the job market.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：职场发展、科技自主、国家战略、个人品质。</t>
+          <t>文章语境：文章讨论政府如何通过监管能力建立对 AI 公司的约束力。
+暗示意思/政治意味/诙谐意味：暗示权力不是喊口号，而来自信息、资源和制度工具。
+特殊考查方式：细节/推理题常用 influence/bargaining power 替换。
+答题技巧：译为“建立筹码/增强制衡能力”更贴政策语境。
+同义替换/错误选项信号：gain leverage; increase bargaining power; strengthen influence
+多场景例句：build leverage over large platforms；build leverage in negotiations；build leverage through better oversight
+其他可用地方：职场谈判、国际关系、政府监管。
+归一化合并：本卡覆盖这些变体：build leverage</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -564,17 +819,28 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>fail-safe</t>
+          <t>build a fail-safe into policy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：失效保护，备用安全机制。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：当主系统失灵时仍能防止严重损失的备份方案。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：工程、风险管理和公共治理常用。</t>
+          <t>字面含义：故障保护机制；失效安全的
+考研核心考点：安全工程和制度设计词
+词汇拆解：fail = 失败；safe = 安全；合起来指失败时仍安全。
+熟词辟义/一词多义：不是“失败是安全的”，而是“即使出故障也能保证安全”。可作名词或形容词。
+语气色彩：技术正式语体。</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：find fail-safes for American export controls。其他国家要准备不被美国管制卡死的备用机制。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：依赖美国比依赖中国好，但单一依赖仍有风险。&lt;br&gt;&lt;b&gt;例句1 个人&lt;/b&gt;：Students need fail-safes, such as backup plans, when preparing for important exams.&lt;br&gt;&lt;b&gt;例句2 经济&lt;/b&gt;：Supply chains need fail-safes against political shocks.&lt;br&gt;&lt;b&gt;例句3 科技&lt;/b&gt;：Critical systems should include fail-safes before they are widely deployed.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：风险管理、考研规划、供应链、科技安全。</t>
+          <t>文章语境：文章指 AI 治理需要在灾难前设计应急机制。
+暗示意思/政治意味/诙谐意味：暗示承认系统会出错，所以要预设保护。
+特殊考查方式：翻译题不要拆成“失败-安全”，译为“故障保护”。
+答题技巧：看到 fail-safe，要想到“预案/保护底线”，不是普通 safety。
+同义替换/错误选项信号：safety backstop; emergency safeguard; backup protection
+多场景例句：a fail-safe mechanism；fail-safe rules for AI systems；build a fail-safe into public policy
+其他可用地方：科技安全、公共安全、风险管理。
+归一化合并：本卡覆盖这些变体：fail-safe</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -586,17 +852,28 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Grammar: The intelligence that... also...</t>
+          <t>when catastrophe strikes</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;结构&lt;/b&gt;：The intelligence + that 定语从句 + also + 谓语。&lt;br&gt;&lt;b&gt;功能&lt;/b&gt;：表达“双刃剑”：同一个特征既制造风险，也创造价值。&lt;br&gt;&lt;b&gt;适合背诵&lt;/b&gt;：科技、教育、社交媒体、基因技术都能套。</t>
+          <t>字面含义：灾难发生/降临
+考研核心考点：新闻体灾难表达
+词汇拆解：catastrophe = 大灾难；strike = 突然袭击/发生
+熟词辟义/一词多义：strike 不只是“打击/罢工”，可指灾难突然发生。
+语气色彩：强负面、新闻感。</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文逻辑&lt;/b&gt;：The intelligence that makes new models dangerous also makes them tremendously useful. 作者承认风险，同时反对简单封锁。&lt;br&gt;&lt;b&gt;例句1 社交媒体&lt;/b&gt;：The connectivity that makes social media distracting also makes it valuable for public communication.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：The pressure that makes exams stressful also makes them a test of discipline.&lt;br&gt;&lt;b&gt;例句3 科技&lt;/b&gt;：The power that makes new technology disruptive also makes it socially valuable.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：考研作文“科技双刃剑”核心句式。</t>
+          <t>文章语境：文章警告不要等灾难发生才制定规则。
+暗示意思/政治意味/诙谐意味：暗示防患于未然的重要性。
+特殊考查方式：熟词僻义：strike = happen suddenly。
+答题技巧：遇到 disaster/catastrophe + strike，译“发生/降临”。
+同义替换/错误选项信号：disaster hits; crisis erupts; calamity occurs
+多场景例句：before catastrophe strikes；when a public-health crisis strikes；if a financial catastrophe hits
+其他可用地方：环境、健康、公共安全。
+归一化合并：本卡覆盖这些变体：catastrophe strikes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -608,17 +885,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rules for supermodels: central argument</t>
+          <t>slapped with export controls</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;中心论点&lt;/b&gt;：前沿 AI 需要监管，但监管应当正式化、专业化、分阶段，并具备国际韧性；不能靠临时拼凑规则、政治交易或狭隘民族主义。</t>
+          <t>字面含义：被突然加上出口管制
+考研核心考点：slap with = 突然强加处罚/限制
+词汇拆解：slap = 拍打；slap A with B = 对 A 强加 B
+熟词辟义/一词多义：slap 熟词僻义：非身体动作，而是政策处罚。
+语气色彩：新闻口吻，带突然和强硬感。</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;可背作文论点&lt;/b&gt;：Powerful technology should be governed by clear rules, expert evaluation and social responsibility.&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Innovation should not be strangled, but it must be guided by rules that protect the public.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A mature society regulates technology before harm becomes irreversible.&lt;br&gt;&lt;b&gt;例句3&lt;/b&gt;：International cooperation is necessary because digital risks rarely stop at national borders.&lt;br&gt;&lt;b&gt;适用话题&lt;/b&gt;：科技生活、道德文明、社会责任、国际合作、经济安全。</t>
+          <t>文章语境：文章指某公司/产品被美国出口管制限制。
+暗示意思/政治意味/诙谐意味：暗示政策动作粗暴、快速、惩罚性。
+特殊考查方式：词义题会用 impose 替换 slapped with。
+答题技巧：译为“被加征/被施加/被突然纳入管制”。
+同义替换/错误选项信号：be hit with; be subject to; be placed under controls
+多场景例句：be slapped with export controls；be slapped with heavy fines；be hit with new sanctions
+其他可用地方：国际贸易、科技竞争、政策风险。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -630,17 +917,28 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>muckraker</t>
+          <t>fears of X were allayed</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：揭黑记者，揭露社会丑闻的人。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻/历史词，带改革时代色彩。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：揭露制度问题、推动公共改革的人。</t>
+          <t>字面含义：对报复/怨恨的担忧被缓解了
+考研核心考点：被动结构 + 抽象名词，考翻译
+词汇拆解：fears = 担忧；grudge = 怨恨/积怨；allay = 缓解
+熟词辟义/一词多义：allay 专接 fear/concern/anxiety，表示减轻担忧。
+语气色彩：正式、新闻语体。</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：muckrakers such as Upton Sinclair 促成 FDA。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：公众监督和媒体揭露能倒逼制度改进。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Muckrakers can force society to confront hidden abuses.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Good journalism should expose problems rather than entertain the public only.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：媒体责任、社会监督、公共伦理。</t>
+          <t>文章语境：文章说明外界担心政策出于私人恩怨，但这种担忧后来减弱。
+暗示意思/政治意味/诙谐意味：暗示政治决策可能被怀疑含有报复动机。
+特殊考查方式：翻译题重点是被动与抽象名词处理。
+答题技巧：可译主动：“这缓解了人们对……的担忧”。
+同义替换/错误选项信号：concerns were eased; fears were dispelled; anxieties were reduced
+多场景例句：fears of a grudge were allayed；concerns about retaliation were eased；public anxiety was allayed
+其他可用地方：政治伦理、公共信任、社会责任。
+归一化合并：本卡覆盖这些变体：Fears of a grudge were allayed</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -652,17 +950,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>bring about</t>
+          <t>de facto ban</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：导致，引起，促成。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：中性，考研高频因果动词短语。&lt;br&gt;&lt;b&gt;区别&lt;/b&gt;：比 cause 更偏“促成某种变化/结果”。</t>
+          <t>字面含义：事实上的禁令
+考研核心考点：法律/政策高频：de facto = 实际上的
+词汇拆解：de facto 来自拉丁语，反义 de jure = 法律上的。
+熟词辟义/一词多义：表示形式上未禁止，效果上等于禁止。
+语气色彩：正式、法律政治语体。</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Pressure from muckrakers brought about the FDA。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Education can bring about long-term social change.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Technological progress may bring about new ethical problems.&lt;br&gt;&lt;b&gt;例句3&lt;/b&gt;：Public pressure can bring about better environmental rules.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：因果论证、教育、环境、科技。</t>
+          <t>文章语境：文章说某些限制可能构成事实禁令。
+暗示意思/政治意味/诙谐意味：暗示政策名义与实际效果不一致。
+特殊考查方式：推理题会考“实际影响”而非字面政策名称。
+答题技巧：看到 de facto，选项里 in effect/in practice 常是替换。
+同义替换/错误选项信号：in effect; in practice; practical ban
+多场景例句：a de facto ban on exports；a de facto monopoly；de facto censorship
+其他可用地方：政策分析、法律、国际贸易。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -674,17 +982,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>capable adviser</t>
+          <t>throughout the past month's brouhaha</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：有能力的顾问。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：不只是能回答问题，而是能提供可操作建议。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：在危险语境中带警惕意味。</t>
+          <t>字面含义：在过去一个月的喧闹争议中
+考研核心考点：brouhaha = 喧嚷/风波，外刊调侃词
+词汇拆解：throughout = 在……整个期间；brouhaha = noisy fuss/controversy
+熟词辟义/一词多义：brouhaha 不是严肃 crisis，而是媒体吵闹和政治喧嚣。
+语气色彩：讽刺、轻微幽默。</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI could become capable advisers to bioterrorists。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：AI 的危险在于能指导行动，而非只提供信息。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：AI can be a capable adviser for students, but it should not replace independent thinking.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A capable adviser helps people make decisions, not merely collect facts.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI、教育学习、道德责任。</t>
+          <t>文章语境：文章用它概括 AI 政策争议的舆论风波。
+暗示意思/政治意味/诙谐意味：暗示争论很热闹，但未必都有实质。
+特殊考查方式：态度题中显示作者略带不耐烦或嘲讽。
+答题技巧：可译“风波/喧嚣/一片吵嚷”，不要译“布鲁哈哈”。
+同义替换/错误选项信号：uproar; fuss; noisy controversy; commotion
+多场景例句：throughout the political brouhaha；amid a media brouhaha；a month-long regulatory brouhaha
+其他可用地方：媒体舆论、政治争议、社会热点。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -696,17 +1014,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>catastrophe strikes</t>
+          <t>buy months, or a year at most</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：灾难降临。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：before catastrophe strikes = 在灾难发生之前。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：强烈、警示，适合风险预防话题。</t>
+          <t>字面含义：但那最多只能争取几个月，或一年时间
+考研核心考点：buy time = 争取时间，熟词僻义
+词汇拆解：buy = 买；buy time = gain time；at most = 最多
+熟词辟义/一词多义：buy 不一定是购买，可指换来/争取。
+语气色彩：转折、现实主义语气。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：regulate the technology before catastrophe strikes。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Governments should act before catastrophe strikes, not after harm is irreversible.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Students should correct bad habits before failure strikes.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技风险、环境保护、健康管理、备考规划。</t>
+          <t>文章语境：文章指出短期限制只能拖延，不能永久解决问题。
+暗示意思/政治意味/诙谐意味：暗示政策窗口很短，根本问题仍需制度化。
+特殊考查方式：翻译题考 buy 的抽象义和 at most。
+答题技巧：that 指前文措施；不要译为“买几个月”。
+同义替换/错误选项信号：gain time; buy a little time; delay the problem temporarily
+多场景例句：buy months, not years；buy time for reform；a measure that buys a year at most
+其他可用地方：政策改革、时间管理、危机应对。
+归一化合并：本卡覆盖这些变体：But that buys months, or a year at most</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -718,17 +1047,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>a row between A and B</t>
+          <t>undesirable</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：A 与 B 之间的争吵/争端。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：row 作名词时可表示争吵，读音不同于 row a boat。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：英式新闻常用。</t>
+          <t>字面含义：不受欢迎的；不合意的；有害的
+考研核心考点：态度评价词，正式负面
+词汇拆解：un- = not；desirable = 值得拥有的/理想的
+熟词辟义/一词多义：desirable 不只是“性感的”，在正式语境中是“可取的”。
+语气色彩：正式、负面但克制。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a row between the company and the Pentagon。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A row between parents and schools can harm students' interests.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：The policy triggered a row between regulators and technology firms.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：新闻阅读、政策争议、教育冲突。</t>
+          <t>文章语境：文章评价某种 AI 释放或限制结果并不可取。
+暗示意思/政治意味/诙谐意味：暗示作者在做政策价值判断。
+特殊考查方式：态度题中是 mild negative。
+答题技巧：选项 harmful/unwelcome/problematic 可替换。
+同义替换/错误选项信号：unwelcome; harmful; problematic; not ideal
+多场景例句：an undesirable outcome；undesirable side effects；socially undesirable consequences
+其他可用地方：科技伦理、健康饮食、社会责任。</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -740,17 +1079,28 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>allay fears</t>
+          <t>improve/increase tremendously</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：缓解担忧，减轻恐惧。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，新闻和政策报道常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：allay concerns / fears / doubts。</t>
+          <t>字面含义：极大地；非常
+考研核心考点：强调副词，用于增强程度
+词汇拆解：tremendous = 巨大的；-ly 副词
+熟词辟义/一词多义：比 very 更正式、更强。
+语气色彩：正式、中性。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Fears of a grudge were allayed。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Clear rules can allay public fears about AI.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Transparent communication helps allay parents' concerns.&lt;br&gt;&lt;b&gt;例句3&lt;/b&gt;：Scientific evidence can allay unnecessary panic.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技治理、教育沟通、公共健康。</t>
+          <t>文章语境：文章用来强调模型能力、影响或变化幅度很大。
+暗示意思/政治意味/诙谐意味：暗示程度不是小变化，而是显著变化。
+特殊考查方式：完形/阅读中可能用 greatly/substantially 替换。
+答题技巧：写作可替换 very much，但别滥用。
+同义替换/错误选项信号：greatly; enormously; substantially; immensely
+多场景例句：improve tremendously；matter tremendously；increase tremendously over time
+其他可用地方：作文：教育进步、科技影响、健康改善。
+归一化合并：本卡覆盖这些变体：tremendously</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -762,17 +1112,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>compel sb to do sth</t>
+          <t>worries about X aside</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：迫使某人做某事。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式、强制性强，比 make sb do 更书面。&lt;br&gt;&lt;b&gt;政治/法律意味&lt;/b&gt;：常用于政府、法律、制度压力。</t>
+          <t>字面含义：撇开对中国的担忧不谈
+考研核心考点：让步/话题转移句首结构
+词汇拆解：aside = 放在一边；A aside = leaving A aside
+熟词辟义/一词多义：aside 不只是“在旁边”，可表示暂且不谈。
+语气色彩：正式、转折引导。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：administration appeared to compel OpenAI to limit access。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Law can compel companies to protect user data.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Exams may compel students to study, but interest keeps them learning.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：法律监管、教育、社会责任。</t>
+          <t>文章语境：文章先让开中国因素，再讨论开放模型本身的问题。
+暗示意思/政治意味/诙谐意味：暗示作者并非只从地缘政治出发，还有更普遍的安全逻辑。
+特殊考查方式：长难句中常作句首状语，容易误判主干。
+答题技巧：先把 aside 结构括起来，再找主句。
+同义替换/错误选项信号：leaving China aside; apart from concerns about China; setting aside geopolitical worries
+多场景例句：worries about privacy aside；cost aside, the plan is sensible；politics aside, the problem remains
+其他可用地方：议论文让步、科技伦理、国际关系。
+归一化合并：本卡覆盖这些变体：Worries about China aside</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -784,17 +1145,28 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>abruptly lift the ban</t>
+          <t>a great lurch in capability</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：突然解除禁令。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：abruptly 暗示决定突兀、缺乏连续性。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：lift a ban / restriction / lockdown。</t>
+          <t>字面含义：一次巨大的猛然跃升/剧烈摇摆
+考研核心考点：lurch = 突然倾斜/猛变，形象词
+词汇拆解：great = 大的；lurch = sudden uncontrolled movement/change
+熟词辟义/一词多义：lurch 可指身体踉跄，也可指政策/技术突然变化。
+语气色彩：形象、负面，强调失控感。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Commerce Department abruptly lifted the ban on Fable。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：政策摇摆，缺乏稳定规则。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A government should not abruptly lift restrictions without explaining its reasons.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Schools should avoid abrupt changes in exam policy.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：政策稳定、公共治理、学校管理。</t>
+          <t>文章语境：文章用它形容模型能力突然释放带来的跃迁。
+暗示意思/政治意味/诙谐意味：暗示变化不是平稳升级，而是突然冲击。
+特殊考查方式：词义题中 sudden shift/jump 可能替换。
+答题技巧：不要译成“伟大的倾斜”，译为“剧烈跃迁/突然摇摆”。
+同义替换/错误选项信号：sudden jump; abrupt shift; uncontrolled swing
+多场景例句：a great lurch in capability；a lurch towards protectionism；a sudden lurch in policy
+其他可用地方：科技变化、经济波动、政策转向。
+归一化合并：本卡覆盖这些变体：a great lurch</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -806,17 +1178,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>fiddle with</t>
+          <t>a sudden jump in capability would unleash chaos</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：摆弄，随手调整。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：略随意，可能暗示小修小改、不够根本。&lt;br&gt;&lt;b&gt;熟词&lt;/b&gt;：fiddle 还可指小提琴，但这里不是。</t>
+          <t>字面含义：每当这些模型最终发布时，能力的突然跃升都会释放混乱
+考研核心考点：时间状语从句 + 强调 did + would 预测后果
+词汇拆解：sudden jump = 突然跃升；capability = 能力；unleash = 释放/引发；chaos = 混乱
+熟词辟义/一词多义：did get released 中 did 强调“确实/最终会”。
+语气色彩：强烈警告、负面预测。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Anthropic fiddled with its safety protections。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：只是调整保护措施就解除禁令，显得监管不严肃。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Do not fiddle with learning methods every day; give one system enough time.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Companies often fiddle with settings instead of solving deeper safety problems.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：学习方法、产品安全、政策批评。</t>
+          <t>文章语境：文章解释为什么长期封锁强模型也会有问题。
+暗示意思/政治意味/诙谐意味：暗示延迟发布会把风险积压，最后集中爆发。
+特殊考查方式：长难句考主干：jump would unleash chaos。
+答题技巧：先删 whenever 从句；did 表强调，不译成“做发布”。
+同义替换/错误选项信号：a sudden jump would unleash chaos; delayed release would cause disruption
+多场景例句：a sudden jump in prices would unleash panic；a sudden jump in capability would disrupt markets；delayed reform may unleash chaos
+其他可用地方：科技治理、经济风险、社会稳定。
+归一化合并：本卡覆盖这些变体：The sudden jump in capability whenever the models did get released would unleash chaos.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -828,17 +1211,28 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>de facto ban</t>
+          <t>build technical expertise</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：事实上的禁令。&lt;br&gt;&lt;b&gt;拉丁词&lt;/b&gt;：de facto = 实际上存在的，不一定写在法律上。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：表面不是禁止，实际效果等于禁止。</t>
+          <t>字面含义：专业知识；专门能力
+考研核心考点：抽象名词，考研高频
+词汇拆解：expert = 专家；-ise/-ise? expertise 名词 = 专业能力
+熟词辟义/一词多义：不可数名词，常搭配 technical/legal/scientific expertise。
+语气色彩：正式、正面。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a wholesale block was a de facto ban。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：High fees can become a de facto ban on poor students entering good schools.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Complex rules may create a de facto barrier to innovation.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育公平、社会政策、科技监管、经济门槛。</t>
+          <t>文章语境：文章强调监管者需要技术专业能力。
+暗示意思/政治意味/诙谐意味：暗示没有专业知识就无法有效监管复杂行业。
+特殊考查方式：细节题常用 knowledge/competence 替换。
+答题技巧：不要加复数；译为“专业知识/专门能力”。
+同义替换/错误选项信号：specialised knowledge; technical competence; professional know-how
+多场景例句：build technical expertise；lack regulatory expertise；draw on scientific expertise
+其他可用地方：学习教育、职场发展、科技治理。
+归一化合并：本卡覆盖这些变体：expertise</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -850,17 +1244,28 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>home market</t>
+          <t>oversight of the overseen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：国内市场，本土市场。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济报道常用。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：一个国家内部需求可支撑企业生存和发展。</t>
+          <t>字面含义：监督 与 被监督对象/被监管
+考研核心考点：同根词对比：oversee/oversight/overseen
+词汇拆解：oversee = 监督；oversight = 监督；overseen = oversee 的过去分词
+熟词辟义/一词多义：oversight 也可指“疏忽”，但监管语境多为“监督”。
+语气色彩：正式、制度语体。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a vast home market would keep China's model-makers going。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：外部封锁不一定有效，因为国内市场足够大。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A large home market can support local innovation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Companies with a strong home market are less vulnerable to foreign pressure.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济发展、科技竞争、国际贸易。</t>
+          <t>文章语境：文章讨论谁来监督 AI 公司，以及监督者如何获得信息。
+暗示意思/政治意味/诙谐意味：暗示监管关系中的信息不对称。
+特殊考查方式：词义题可能考 oversight 的两义。
+答题技巧：看搭配：regulatory oversight = 监管；an oversight = 疏忽。
+同义替换/错误选项信号：supervision; monitoring; scrutiny; regulated entities
+多场景例句：regulatory oversight of AI；companies being overseen by agencies；strengthen oversight without micromanaging
+其他可用地方：公共治理、职场管理、社会责任。
+归一化合并：本卡覆盖这些变体：oversight &amp; overseen</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -872,17 +1277,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>publicly available</t>
+          <t>Ideally &amp; Alas</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：公开可获得的。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，常用于数据、资源、模型、信息。&lt;br&gt;&lt;b&gt;反义&lt;/b&gt;：restricted / private / confidential。</t>
+          <t>字面含义：理想情况下 与 可惜/遗憾的是
+考研核心考点：外刊论证转折标记
+词汇拆解：ideally = 理想情况下；alas = 可惜/唉
+熟词辟义/一词多义：alas 带老派、轻微戏谑或无奈语气。
+语气色彩：先设理想，再指出现实不足。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a gulf between publicly available and restricted models。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Publicly available educational resources can reduce inequality.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Not all publicly available information is reliable.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育资源、信息素养、AI 模型、公共服务。</t>
+          <t>文章语境：文章可能用 Ideally 提方案，用 Alas 转向现实约束。
+暗示意思/政治意味/诙谐意味：暗示作者结构：理想方案 vs 现实困境。
+特殊考查方式：阅读结构题可定位转折。
+答题技巧：看到 Alas，后面往往是坏消息或限制条件。
+同义替换/错误选项信号：in an ideal world; unfortunately; regrettably; sadly
+多场景例句：Ideally, regulators would act early; alas, politics intervenes；Ideally, standards would be clear; alas, they remain vague；Ideally, firms would self-regulate; alas, incentives differ
+其他可用地方：议论文结构、作文让步转折。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -894,17 +1309,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>unleash chaos</t>
+          <t>immense sovereign power</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：释放混乱，引发大乱。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：强烈，unleash 暗示把原本被压住的力量放出来。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：unleash creativity / violence / chaos / potential。</t>
+          <t>字面含义：巨大的主权权力
+考研核心考点：政治经济类立场词
+词汇拆解：immense = 巨大的；sovereign = 主权的/至高的；power = 权力/强权
+熟词辟义/一词多义：power 在政治语境中不是电力/能力，而是权力、政权或强制力。
+语气色彩：正式、强政治色彩。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：能力突然跃升 would unleash chaos。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A sudden release of powerful technology may unleash chaos.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Poorly planned reforms can unleash confusion in schools.&lt;br&gt;&lt;b&gt;例句3&lt;/b&gt;：Education should unleash potential, not anxiety.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技风险、教育改革、社会治理、个人潜能。</t>
+          <t>文章语境：文章指国家在管制技术和贸易时拥有极大主权权力。
+暗示意思/政治意味/诙谐意味：暗示政府可强制执行规则，但也可能滥用。
+特殊考查方式：推理题会考是正当治理还是霸权/过度干预。
+答题技巧：看到 sovereign，联想到国家主权、独立、最高权威。
+同义替换/错误选项信号：vast state power; sovereign authority; supreme governmental power
+多场景例句：exercise immense sovereign power；limit immense sovereign power；immense sovereign power over trade
+其他可用地方：国际关系、政府监管、公共权力边界。</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -916,17 +1341,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>trusted institutions</t>
+          <t>strategic interest</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：可信机构。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：被认为有能力、有责任、有规则约束的组织。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政策/治理语境常用。</t>
+          <t>字面含义：战略利益
+考研核心考点：国际关系/经济类高频名词短语
+词汇拆解：strategic = 战略性的；interest = 利益/关切，不是兴趣
+熟词辟义/一词多义：interest 在政治经济中常译“利益”，复数 interests 更明显。
+语气色彩：正式、国家政策语体。</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：staggered release to trusted institutions。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：不是所有人立刻使用，而是先给有责任能力的机构。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Sensitive data should be shared only with trusted institutions.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Universities can serve as trusted institutions in public debates.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：AI 安全、公共卫生、教育机构、社会信任。</t>
+          <t>文章语境：文章说明 AI 管制与国家战略利益相关。
+暗示意思/政治意味/诙谐意味：暗示政策不只是商业选择，而涉及安全和长期竞争。
+特殊考查方式：选项中 national security concern/economic benefit 可能替换。
+答题技巧：interest 若在国家/政府语境，优先译“利益”。
+同义替换/错误选项信号：national interest; strategic concern; long-term security interest
+多场景例句：protect a strategic interest；serve national strategic interests；a strategic interest in advanced technology
+其他可用地方：国际关系、科技强国、经济安全。</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -938,17 +1373,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>risk to tolerate</t>
+          <t>indiscriminate tariffs</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：可容忍的风险。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：how much risk to tolerate。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政策决策词，强调价值判断。</t>
+          <t>字面含义：无差别关税；不加区分的关税
+考研核心考点：经济政策负面搭配
+词汇拆解：in- 否定；discriminate = 区分；tariffs = 关税
+熟词辟义/一词多义：discriminate 既可指区分，也可指歧视；indiscriminate = 不加选择的。
+语气色彩：批评性，暗示粗暴和低效。</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：how much risk to tolerate belongs to elected leaders。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：技术专家能评估风险，但社会能接受多少风险是政治问题。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A society must decide how much risk to tolerate in exchange for innovation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Students should know how much risk to tolerate when choosing a career path.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技伦理、职业选择、公共政策。</t>
+          <t>文章语境：文章把粗糙贸易手段与更精准的 AI 政策相对照。
+暗示意思/政治意味/诙谐意味：暗示作者反对一刀切式贸易政策。
+特殊考查方式：态度题中 negative 信号明显。
+答题技巧：impose indiscriminate tariffs = 无差别加征关税。
+同义替换/错误选项信号：blanket tariffs; across-the-board tariffs; arbitrary duties
+多场景例句：impose indiscriminate tariffs；indiscriminate tariffs on imports；avoid blanket trade restrictions
+其他可用地方：经济生活、国际贸易、政策批判。</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1044,7 +1489,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>英语::外刊精读</t>
+          <t>考研英语::外刊精读</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-08-02 02:03:56
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/Rules for supermodels/anki/anki.xlsx
@@ -43,7 +43,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：从灾难中产生/走出来
 &lt;b&gt;考研核心考点&lt;/b&gt;：灾难后的制度或经验产物
-&lt;b&gt;词汇拆解&lt;/b&gt;：come out of = emerge from/result from；disasters = crises/calamities｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：come out of + disaster/crisis。中文：come out of 从“走出来”引申为“由……产生”。English: `come out of X` can mean `emerge from` or `result from X`.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：come out of 不只是“出来”，还可表示“由……产生”。
 &lt;b&gt;语气色彩&lt;/b&gt;：中性偏正式，常用于历史经验、制度改革。</t>
         </is>
@@ -55,13 +55,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：主旨/推理题会考“某制度为何出现”。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 come out of + 抽象/负面事件，优先译成“源于/产生于”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：emerge from; result from; be born of; grow out of
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Useful rules often come out of disasters that expose old weaknesses. 译：有用的规则往往产生于暴露旧弱点的灾难。&lt;br&gt;2. In an exam passage, `come out of disasters/crises` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`come out of disasters/crises` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `come out of disasters/crises` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `come out of disasters/crises` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Useful rules often come out of disasters that expose old weaknesses. 译：有用的规则往往产生于暴露旧弱点的灾难。&lt;br&gt;2. Better safety standards can come out of crises if society learns from failure. 译：如果社会能从失败中学习，更好的安全标准就可能从危机中产生。&lt;br&gt;3. Some public-health reforms came out of disasters that revealed weak institutions. 译：一些公共卫生改革源于暴露制度薄弱的灾难。
 &lt;b&gt;其他可用地方&lt;/b&gt;：社会责任、科技治理、公共安全。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：come out of disasters
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：从灾难中产生/走出来。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：come out of 不只是“出来”，还可表示“由……产生”。 例：The expression `come out of disasters/crises` should be interpreted through its context. 译：表达 `come out of disasters/crises` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：come out of disasters/crises；本卡覆盖这些变体：come out of disasters
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：从灾难中产生/走出来。例：Useful rules often come out of disasters that expose old weaknesses. 译：有用的规则往往产生于暴露旧弱点的灾难。 2. 文章义/考试义：come out of 不只是“出来”，还可表示“由……产生”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Useful rules often come out of disasters that expose old weaknesses. 译：有用的规则往往产生于暴露旧弱点的灾难。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Better safety standards can come out of crises if society learns from failure. 译：如果社会能从失败中学习，更好的安全标准就可能从危机中产生。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -80,7 +79,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：大灾难；严重灾祸
 &lt;b&gt;考研核心考点&lt;/b&gt;：比 disaster 更书面、更严重的负面名词
-&lt;b&gt;词汇拆解&lt;/b&gt;：calam- 无需死背；常搭配 natural/political/economic calamity｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：calam- 无需死背；常搭配 natural/political/economic calamity。中文：这是一个固定搭配或外刊表达，本卡重点是把 `avert a calamity` 和“大灾难；严重灾祸”一起记，尤其注意搭配对象和语境义。English: `avert a calamity` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `大灾难；严重灾祸` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：可指具体灾害，也可指抽象灾难性后果。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、强负面。</t>
         </is>
@@ -92,13 +91,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中常指作者担忧或警惕。
 &lt;b&gt;答题技巧&lt;/b&gt;：遇到 calamity 不要译轻，选项里 catastrophe/crisis 常是替换。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：catastrophe; disaster; crisis; debacle
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Responsible regulation can help society avert a calamity before it happens. 译：负责任的监管能够帮助社会在灾难发生前避免灾难。&lt;br&gt;2. In an exam passage, `avert a calamity` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`avert a calamity` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `avert a calamity` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `avert a calamity` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Responsible regulation can help society avert a calamity before it happens. 译：负责任的监管能够帮助社会在灾难发生前避免灾难。&lt;br&gt;2. Public institutions should consider how avert a calamity affects fairness, efficiency and trust. 译：公共机构应考虑 avert a calamity 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss avert a calamity without ignoring long-term responsibility. 译：一个成熟社会可以讨论 avert a calamity，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：环境灾害、公共安全、科技风险。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：calamity
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：大灾难；严重灾祸。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：可指具体灾害，也可指抽象灾难性后果。 例：The expression `avert a calamity` should be interpreted through its context. 译：表达 `avert a calamity` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：avert a calamity；本卡覆盖这些变体：calamity
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：大灾难；严重灾祸。例：Responsible regulation can help society avert a calamity before it happens. 译：负责任的监管能够帮助社会在灾难发生前避免灾难。 2. 文章义/考试义：可指具体灾害，也可指抽象灾难性后果。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Responsible regulation can help society avert a calamity before it happens. 译：负责任的监管能够帮助社会在灾难发生前避免灾难。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how avert a calamity affects fairness, efficiency and trust. 译：公共机构应考虑 avert a calamity 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -117,7 +115,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：自愿性标准
 &lt;b&gt;考研核心考点&lt;/b&gt;：政策类阅读常见：非强制监管工具
-&lt;b&gt;词汇拆解&lt;/b&gt;：voluntary = 自愿的；standards = standards/rules/benchmarks｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：voluntary = 自愿的；standards = standards/rules/benchmarks。中文：这是一个固定搭配或外刊表达，本卡重点是把 `voluntary standards` 和“自愿性标准”一起记，尤其注意搭配对象和语境义。English: `voluntary standards` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `自愿性标准` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：standard 不只是“标准答案”，还指行业规范。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性，但常暗示约束力不足。</t>
         </is>
@@ -129,12 +127,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会问措施性质：mandatory 还是 voluntary。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 voluntary standards，要留意作者是否认为其 too weak。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：self-imposed rules; non-binding guidelines; industry standards
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Voluntary standards are useful, but they cannot replace clear public rules. 译：自愿性标准有用，但不能取代明确的公共规则。&lt;br&gt;2. In an exam passage, `voluntary standards` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`voluntary standards` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `voluntary standards` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `voluntary standards` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Voluntary standards are useful, but they cannot replace clear public rules. 译：自愿性标准有用，但不能取代明确的公共规则。&lt;br&gt;2. Clear public rules can make voluntary standards safer and more accountable. 译：清晰的公共规则可以让 voluntary standards 更安全、更可问责。&lt;br&gt;3. Without social responsibility, voluntary standards may create risks that spread beyond one company. 译：如果缺乏社会责任，voluntary standards 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技监管、企业责任、行业自律。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：自愿性标准。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：standard 不只是“标准答案”，还指行业规范。 例：The expression `voluntary standards` should be interpreted through its context. 译：表达 `voluntary standards` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：voluntary standards
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：自愿性标准。例：Voluntary standards are useful, but they cannot replace clear public rules. 译：自愿性标准有用，但不能取代明确的公共规则。 2. 文章义/考试义：standard 不只是“标准答案”，还指行业规范。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Voluntary standards are useful, but they cannot replace clear public rules. 译：自愿性标准有用，但不能取代明确的公共规则。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make voluntary standards safer and more accountable. 译：清晰的公共规则可以让 voluntary standards 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -153,7 +150,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：被护栏限制的；设有安全边界的
 &lt;b&gt;考研核心考点&lt;/b&gt;：科技语境中的新用法：给系统加安全限制
-&lt;b&gt;词汇拆解&lt;/b&gt;：guardrail = 护栏/防护栏；-ed 表示“被设置防护”。｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：guardrail = 护栏/防护栏；-ed 表示“被设置防护”。。中文：这是一个可替换词组，本卡重点是把 `guardrail a model / a guardrailed release` 和“被护栏限制的；设有安全边界的”一起记，尤其注意搭配对象和语境义。English: `guardrail a model / a guardrailed release` functions as a interchangeable phrase pattern; learn the whole chunk with its meaning `被护栏限制的；设有安全边界的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：guardrail 从道路护栏引申为政策/技术边界。
 &lt;b&gt;语气色彩&lt;/b&gt;：技术政策语体，中性偏谨慎。</t>
         </is>
@@ -165,14 +162,13 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能考从具体护栏到抽象安全边界。
 &lt;b&gt;答题技巧&lt;/b&gt;：译成“设有安全护栏/受安全限制”，不要死译成“有栏杆的”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：safeguarded; constrained; safety-bounded
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Developers should guardrail a model before releasing it to the public. 译：开发者在向公众发布模型之前应当为模型设置安全护栏。&lt;br&gt;2. In an exam passage, `guardrail a model / a guardrailed release` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`guardrail a model / a guardrailed release` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `guardrail a model / a guardrailed release` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `guardrail a model / a guardrailed release` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Developers should guardrail a model before releasing it to the public. 译：开发者在向公众发布模型之前应当为模型设置安全护栏。&lt;br&gt;2. Clear public rules can make guardrail a model safer and more accountable. 译：清晰的公共规则可以让 guardrail a model 更安全、更可问责。&lt;br&gt;3. Without social responsibility, guardrail a model may create risks that spread beyond one company. 译：如果缺乏社会责任，guardrail a model 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、AI 安全、制度设计。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：guardrailed
 &lt;b&gt;归一化合并&lt;/b&gt;：原表达 `a guardrailed release / guardrail a model` 已改为考研一可迁移原型 `guardrail a model / a guardrailed release`。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：被护栏限制的；设有安全边界的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：guardrail 从道路护栏引申为政策/技术边界。 例：The expression `guardrail a model / a guardrailed release` should be interpreted through its context. 译：表达 `guardrail a model / a guardrailed release` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：guardrail a model / a guardrailed release；本卡覆盖这些变体：guardrailed
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：被护栏限制的；设有安全边界的。例：Developers should guardrail a model before releasing it to the public. 译：开发者在向公众发布模型之前应当为模型设置安全护栏。 2. 文章义/考试义：guardrail 从道路护栏引申为政策/技术边界。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Developers should guardrail a model before releasing it to the public. 译：开发者在向公众发布模型之前应当为模型设置安全护栏。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make guardrail a model safer and more accountable. 译：清晰的公共规则可以让 guardrail a model 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -191,7 +187,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：出口管制
 &lt;b&gt;考研核心考点&lt;/b&gt;：国际关系/科技竞争高频政策词
-&lt;b&gt;词汇拆解&lt;/b&gt;：export = 出口；controls = 管制措施｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：export = 出口；controls = 管制措施。中文：这是一个固定搭配或外刊表达，本卡重点是把 `export controls` 和“出口管制”一起记，尤其注意搭配对象和语境义。English: `export controls` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `出口管制` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：control 在政策语境中多译为“管制/限制”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、政治经济色彩强。</t>
         </is>
@@ -203,12 +199,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会用 restrictions/curbs 替换 controls。
 &lt;b&gt;答题技巧&lt;/b&gt;：遇到 export controls，定位政府干预与战略利益。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：export restrictions; trade curbs; technology controls
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Export controls can protect national security but may also slow global cooperation. 译：出口管制可以保护国家安全，但也可能减缓全球合作。&lt;br&gt;2. In an exam passage, `export controls` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`export controls` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `export controls` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `export controls` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Export controls can protect national security but may also slow global cooperation. 译：出口管制可以保护国家安全，但也可能减缓全球合作。&lt;br&gt;2. Public institutions should consider how export controls affects fairness, efficiency and trust. 译：公共机构应考虑 export controls 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss export controls without ignoring long-term responsibility. 译：一个成熟社会可以讨论 export controls，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技竞争、国际贸易、国家安全。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：出口管制。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：control 在政策语境中多译为“管制/限制”。 例：The expression `export controls` should be interpreted through its context. 译：表达 `export controls` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：export controls
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：出口管制。例：Export controls can protect national security but may also slow global cooperation. 译：出口管制可以保护国家安全，但也可能减缓全球合作。 2. 文章义/考试义：control 在政策语境中多译为“管制/限制”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Export controls can protect national security but may also slow global cooperation. 译：出口管制可以保护国家安全，但也可能减缓全球合作。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how export controls affects fairness, efficiency and trust. 译：公共机构应考虑 export controls 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -227,7 +222,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：临时编规则；边做边定规则
 &lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语：on the fly = 即时地、临场地
-&lt;b&gt;词汇拆解&lt;/b&gt;：make up = 编造/制定；rules = 规则；on the fly = without prior planning｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：make up = 编造/制定；rules = 规则；on the fly = without prior planning。中文：这是一个固定搭配或外刊表达，本卡重点是把 `make up rules on the fly` 和“临时编规则；边做边定规则”一起记，尤其注意搭配对象和语境义。English: `make up rules on the fly` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `临时编规则；边做边定规则` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：make up 不只是“化妆/组成”，可指“编造、临时凑出”。
 &lt;b&gt;语气色彩&lt;/b&gt;：口语化、批评性，暗示缺乏制度性。</t>
         </is>
@@ -239,12 +234,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中是负面信号。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 on the fly，理解为“临时/即时”，不是“在飞行中”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：improvise rules; ad-lib regulations; set rules case by case
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Governments should not make up rules on the fly when powerful technology is involved. 译：当涉及强大技术时，政府不应临时编规则。&lt;br&gt;2. In an exam passage, `make up rules on the fly` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`make up rules on the fly` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `make up rules on the fly` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `make up rules on the fly` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Governments should not make up rules on the fly when powerful technology is involved. 译：当涉及强大技术时，政府不应临时编规则。&lt;br&gt;2. Clear public rules can make make up rules on the fly safer and more accountable. 译：清晰的公共规则可以让 make up rules on the fly 更安全、更可问责。&lt;br&gt;3. Without social responsibility, make up rules on the fly may create risks that spread beyond one company. 译：如果缺乏社会责任，make up rules on the fly 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技治理、公共管理、制度建设。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：临时编规则；边做边定规则。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：make up 不只是“化妆/组成”，可指“编造、临时凑出”。 例：The expression `make up rules on the fly` should be interpreted through its context. 译：表达 `make up rules on the fly` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：make up rules on the fly
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：临时编规则；边做边定规则。例：Governments should not make up rules on the fly when powerful technology is involved. 译：当涉及强大技术时，政府不应临时编规则。 2. 文章义/考试义：make up 不只是“化妆/组成”，可指“编造、临时凑出”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Governments should not make up rules on the fly when powerful technology is involved. 译：当涉及强大技术时，政府不应临时编规则。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make make up rules on the fly safer and more accountable. 译：清晰的公共规则可以让 make up rules on the fly 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -263,7 +257,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：民族主义色彩；国家主义意味
 &lt;b&gt;考研核心考点&lt;/b&gt;：态度与立场词：tinge 表示淡淡的色彩/倾向
-&lt;b&gt;词汇拆解&lt;/b&gt;：nationalistic = 民族主义的；tinge = slight trace/color｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：nationalistic = 民族主义的；tinge = slight trace/color。中文：这是一个固定搭配或外刊表达，本卡重点是把 `nationalistic tinge` 和“民族主义色彩；国家主义意味”一起记，尤其注意搭配对象和语境义。English: `nationalistic tinge` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `民族主义色彩；国家主义意味` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：tinge 可指颜色，也可指情绪、政治色彩。
 &lt;b&gt;语气色彩&lt;/b&gt;：含蓄批评，journalistic。</t>
         </is>
@@ -275,12 +269,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：推理题可能问作者如何看待政策动机。
 &lt;b&gt;答题技巧&lt;/b&gt;：不要译成“民族颜色”，应译为“民族主义意味”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：nationalist flavour; patriotic colouring; political undertone
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A nationalistic tinge can make a technical debate more emotional and less rational. 译：民族主义色彩会让技术争论更加情绪化、较少理性。&lt;br&gt;2. In an exam passage, `nationalistic tinge` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`nationalistic tinge` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `nationalistic tinge` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `nationalistic tinge` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A nationalistic tinge can make a technical debate more emotional and less rational. 译：民族主义色彩会让技术争论更加情绪化、较少理性。&lt;br&gt;2. Public institutions should consider how nationalistic tinge affects fairness, efficiency and trust. 译：公共机构应考虑 nationalistic tinge 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss nationalistic tinge without ignoring long-term responsibility. 译：一个成熟社会可以讨论 nationalistic tinge，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：国际关系、科技竞争、政治态度。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：民族主义色彩；国家主义意味。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：tinge 可指颜色，也可指情绪、政治色彩。 例：The expression `nationalistic tinge` should be interpreted through its context. 译：表达 `nationalistic tinge` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：nationalistic tinge
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：民族主义色彩；国家主义意味。例：A nationalistic tinge can make a technical debate more emotional and less rational. 译：民族主义色彩会让技术争论更加情绪化、较少理性。 2. 文章义/考试义：tinge 可指颜色，也可指情绪、政治色彩。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A nationalistic tinge can make a technical debate more emotional and less rational. 译：民族主义色彩会让技术争论更加情绪化、较少理性。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how nationalistic tinge affects fairness, efficiency and trust. 译：公共机构应考虑 nationalistic tinge 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -299,7 +292,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：优先于；凌驾于
 &lt;b&gt;考研核心考点&lt;/b&gt;：写作高分逻辑短语：表达价值排序
-&lt;b&gt;词汇拆解&lt;/b&gt;：precedence = priority；take precedence over A = be more important than A｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：take + precedence + over。中文：precedence = 优先权，over 后接被放在次要位置的对象。English: `take precedence over X` means `be treated as more important than X`.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：precedence 与 precedent 不同：前者优先权，后者先例。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性。</t>
         </is>
@@ -311,12 +304,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题常考抽象名词的主谓搭配。
 &lt;b&gt;答题技巧&lt;/b&gt;：选项里 priority/come before 常是同义替换。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：come before; outweigh; be given priority over
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Public safety should take precedence over short-term commercial gains. 译：公共安全应当优先于短期商业利益。&lt;br&gt;2. In an exam passage, `take precedence over` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`take precedence over` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `take precedence over` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `take precedence over` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Public safety should take precedence over short-term commercial gains. 译：公共安全应当优先于短期商业利益。&lt;br&gt;2. In education policy, equal access should take precedence over narrow competition. 译：在教育政策中，公平机会应当优先于狭隘竞争。&lt;br&gt;3. Environmental responsibility must take precedence over unchecked industrial expansion. 译：环境责任必须优先于不受约束的工业扩张。
 &lt;b&gt;其他可用地方&lt;/b&gt;：作文：社会责任、科技伦理、公共利益。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：优先于；凌驾于。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：precedence 与 precedent 不同：前者优先权，后者先例。 例：The expression `take precedence over` should be interpreted through its context. 译：表达 `take precedence over` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：take precedence over
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：优先于；凌驾于。例：Public safety should take precedence over short-term commercial gains. 译：公共安全应当优先于短期商业利益。 2. 文章义/考试义：precedence 与 precedent 不同：前者优先权，后者先例。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Public safety should take precedence over short-term commercial gains. 译：公共安全应当优先于短期商业利益。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：In education policy, equal access should take precedence over narrow competition. 译：在教育政策中，公平机会应当优先于狭隘竞争。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -335,7 +327,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：前沿人工智能；最先进 AI
 &lt;b&gt;考研核心考点&lt;/b&gt;：科技类核心术语
-&lt;b&gt;词汇拆解&lt;/b&gt;：frontier = 边界/前沿；AI = artificial intelligence｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：frontier = 边界/前沿；AI = artificial intelligence。中文：这是一个名词短语，本卡重点是把 `frontier AI models` 和“前沿人工智能；最先进 AI”一起记，尤其注意搭配对象和语境义。English: `frontier AI models` functions as a noun phrase; learn the whole chunk with its meaning `前沿人工智能；最先进 AI` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：frontier 不只是“边疆”，也指研究或技术最前沿。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、技术政策语体。</t>
         </is>
@@ -347,13 +339,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会用 cutting-edge/advanced 替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：翻译时加“前沿/最先进”，不要译成“边境 AI”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：advanced AI; cutting-edge AI; state-of-the-art models
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Frontier AI models require oversight because their abilities are still uncertain. 译：前沿人工智能模型需要监管，因为它们的能力仍然不确定。&lt;br&gt;2. In an exam passage, `frontier AI models` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`frontier AI models` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `frontier AI models` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `frontier AI models` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Frontier AI models require oversight because their abilities are still uncertain. 译：前沿人工智能模型需要监管，因为它们的能力仍然不确定。&lt;br&gt;2. Clear public rules can make frontier AI models safer and more accountable. 译：清晰的公共规则可以让 frontier AI models 更安全、更可问责。&lt;br&gt;3. Without social responsibility, frontier AI models may create risks that spread beyond one company. 译：如果缺乏社会责任，frontier AI models 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、AI 治理、创新与安全。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：frontier AI
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：前沿人工智能；最先进 AI。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：frontier 不只是“边疆”，也指研究或技术最前沿。 例：The expression `frontier AI models` should be interpreted through its context. 译：表达 `frontier AI models` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：frontier AI models；本卡覆盖这些变体：frontier AI
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：前沿人工智能；最先进 AI。例：Frontier AI models require oversight because their abilities are still uncertain. 译：前沿人工智能模型需要监管，因为它们的能力仍然不确定。 2. 文章义/考试义：frontier 不只是“边疆”，也指研究或技术最前沿。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Frontier AI models require oversight because their abilities are still uncertain. 译：前沿人工智能模型需要监管，因为它们的能力仍然不确定。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make frontier AI models safer and more accountable. 译：清晰的公共规则可以让 frontier AI models 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -372,7 +363,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：开放权重的
 &lt;b&gt;考研核心考点&lt;/b&gt;：AI 术语：模型参数可公开获取/下载
-&lt;b&gt;词汇拆解&lt;/b&gt;：open = 开放；weight = 模型权重/参数，不是体重。｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：open = 开放；weight = 模型权重/参数，不是体重。。中文：这是一个名词短语，本卡重点是把 `open-weight AI models` 和“开放权重的”一起记，尤其注意搭配对象和语境义。English: `open-weight AI models` functions as a noun phrase; learn the whole chunk with its meaning `开放权重的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：weight 在 AI 中指参数；熟词僻义很关键。
 &lt;b&gt;语气色彩&lt;/b&gt;：技术语体，中性但政策敏感。</t>
         </is>
@@ -384,13 +375,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能考 weight 的技术义。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 open-weight，要想到可复制、可改造、难封禁。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：open-source-like models; publicly available weights
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Open-weight AI models can spread quickly once their parameters are released. 译：开放权重的人工智能模型一旦参数发布，就会迅速传播。&lt;br&gt;2. In an exam passage, `open-weight AI models` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`open-weight AI models` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `open-weight AI models` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `open-weight AI models` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Open-weight AI models can spread quickly once their parameters are released. 译：开放权重的人工智能模型一旦参数发布，就会迅速传播。&lt;br&gt;2. Clear public rules can make open-weight AI models safer and more accountable. 译：清晰的公共规则可以让 open-weight AI models 更安全、更可问责。&lt;br&gt;3. Without social responsibility, open-weight AI models may create risks that spread beyond one company. 译：如果缺乏社会责任，open-weight AI models 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技创新、开放知识、风险治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：open-weight
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：开放权重的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：weight 在 AI 中指参数；熟词僻义很关键。 例：The expression `open-weight AI models` should be interpreted through its context. 译：表达 `open-weight AI models` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：open-weight AI models；本卡覆盖这些变体：open-weight
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：开放权重的。例：Open-weight AI models can spread quickly once their parameters are released. 译：开放权重的人工智能模型一旦参数发布，就会迅速传播。 2. 文章义/考试义：weight 在 AI 中指参数；熟词僻义很关键。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Open-weight AI models can spread quickly once their parameters are released. 译：开放权重的人工智能模型一旦参数发布，就会迅速传播。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make open-weight AI models safer and more accountable. 译：清晰的公共规则可以让 open-weight AI models 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -409,7 +399,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：摆弄/篡改了它的安全保护
 &lt;b&gt;考研核心考点&lt;/b&gt;：fiddle with = 胡乱改动，语气比 modify 更轻佻
-&lt;b&gt;词汇拆解&lt;/b&gt;：fiddle = 摆弄；safety protections = 安全保护措施｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：fiddle = 摆弄；safety protections = 安全保护措施。中文：这是一个可替换词组，本卡重点是把 `tinker/fiddle with safety protections` 和“摆弄/篡改了它的安全保护”一起记，尤其注意搭配对象和语境义。English: `tinker/fiddle with safety protections` functions as a interchangeable phrase pattern; learn the whole chunk with its meaning `摆弄/篡改了它的安全保护` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：fiddle with 常暗示不专业或不该改。
 &lt;b&gt;语气色彩&lt;/b&gt;：批评、带轻微调侃。</t>
         </is>
@@ -421,13 +411,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题可判断作者担心滥用。
 &lt;b&gt;答题技巧&lt;/b&gt;：译为“乱改/摆弄”，不要中性译为“调整”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：tamper with; tinker with; mess with; alter
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Users may tinker with safety protections if a system is too easy to modify. 译：如果系统太容易修改，用户可能会摆弄其安全保护。&lt;br&gt;2. In an exam passage, `tinker/fiddle with safety protections` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`tinker/fiddle with safety protections` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `tinker/fiddle with safety protections` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `tinker/fiddle with safety protections` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Users may tinker with safety protections if a system is too easy to modify. 译：如果系统太容易修改，用户可能会摆弄其安全保护。&lt;br&gt;2. Public institutions should consider how tinker/fiddle with safety protections affects fairness, efficiency and trust. 译：公共机构应考虑 tinker/fiddle with safety protections 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss tinker/fiddle with safety protections without ignoring long-term responsibility. 译：一个成熟社会可以讨论 tinker/fiddle with safety protections，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技安全、个人责任、平台治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：tinker with；fiddled with its safety protections；tinker with them
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：摆弄/篡改了它的安全保护。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：fiddle with 常暗示不专业或不该改。 例：The expression `tinker/fiddle with safety protections` should be interpreted through its context. 译：表达 `tinker/fiddle with safety protections` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：tinker/fiddle with safety protections；本卡覆盖这些变体：tinker with；fiddled with its safety protections；tinker with them
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：摆弄/篡改了它的安全保护。例：Users may tinker with safety protections if a system is too easy to modify. 译：如果系统太容易修改，用户可能会摆弄其安全保护。 2. 文章义/考试义：fiddle with 常暗示不专业或不该改。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Users may tinker with safety protections if a system is too easy to modify. 译：如果系统太容易修改，用户可能会摆弄其安全保护。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how tinker/fiddle with safety protections affects fairness, efficiency and trust. 译：公共机构应考虑 tinker/fiddle with safety protections 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -446,7 +435,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：严厉打击知识蒸馏/能力提炼
 &lt;b&gt;考研核心考点&lt;/b&gt;：科技监管 + 熟词僻义组合
-&lt;b&gt;词汇拆解&lt;/b&gt;：crack down on = 严打；distillation = AI 知识蒸馏/能力提炼｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：crack down on + object。中文：on 后面是被严厉打击的对象，本卡重点是 `distillation` 这种技术绕道。English: `crack down on X` means `take strict action against X`.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：distillation 不是化学蒸馏，而是模型能力转移。
 &lt;b&gt;语气色彩&lt;/b&gt;：强监管、技术敏感。</t>
         </is>
@@ -458,13 +447,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题问政府措施时，该短语是定位点。
 &lt;b&gt;答题技巧&lt;/b&gt;：不要死译“打击蒸馏”，要译“整治知识蒸馏/能力转移”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：clamp down on model distillation; curb capability extraction; restrict knowledge transfer
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators may crack down on distillation if it helps firms bypass restrictions. 译：如果知识蒸馏帮助企业绕过限制，监管者可能会对此进行打击。&lt;br&gt;2. In an exam passage, `crack down on distillation` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`crack down on distillation` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `crack down on distillation` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `crack down on distillation` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators may crack down on distillation if it helps firms bypass restrictions. 译：如果知识蒸馏帮助企业绕过限制，监管者可能会对此进行打击。&lt;br&gt;2. Public institutions should consider how crack down on distillation affects fairness, efficiency and trust. 译：公共机构应考虑 crack down on distillation 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss crack down on distillation without ignoring long-term responsibility. 译：一个成熟社会可以讨论 crack down on distillation，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：AI 安全、知识产权、科技治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：crack down on；cracking down on distillation
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：严厉打击知识蒸馏/能力提炼。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：distillation 不是化学蒸馏，而是模型能力转移。 例：The expression `crack down on distillation` should be interpreted through its context. 译：表达 `crack down on distillation` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：crack down on distillation；本卡覆盖这些变体：crack down on；cracking down on distillation
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：严厉打击知识蒸馏/能力提炼。例：Regulators may crack down on distillation if it helps firms bypass restrictions. 译：如果知识蒸馏帮助企业绕过限制，监管者可能会对此进行打击。 2. 文章义/考试义：distillation 不是化学蒸馏，而是模型能力转移。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Regulators may crack down on distillation if it helps firms bypass restrictions. 译：如果知识蒸馏帮助企业绕过限制，监管者可能会对此进行打击。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how crack down on distillation affects fairness, efficiency and trust. 译：公共机构应考虑 crack down on distillation 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -483,7 +471,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：行不通的；不可操作的
 &lt;b&gt;考研核心考点&lt;/b&gt;：政策评价词，强烈负面
-&lt;b&gt;词汇拆解&lt;/b&gt;：un- = not；workable = 可行的｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：un- = not；workable = 可行的。中文：这是一个名词短语，本卡重点是把 `an unworkable regulatory scheme` 和“行不通的；不可操作的”一起记，尤其注意搭配对象和语境义。English: `an unworkable regulatory scheme` functions as a noun phrase; learn the whole chunk with its meaning `行不通的；不可操作的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：workable 不是“能工作的”，而是“可执行/可操作”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、批评性。</t>
         </is>
@@ -495,13 +483,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 negative/critical。
 &lt;b&gt;答题技巧&lt;/b&gt;：选项 feasible/practical 是反义，impractical 是同义。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：impractical; infeasible; impossible to enforce
-&lt;b&gt;多场景例句&lt;/b&gt;：1. An unworkable regulatory scheme may look strict but fail in practice. 译：一套不可操作的监管方案看起来严格，但在实践中可能失败。&lt;br&gt;2. In an exam passage, `an unworkable regulatory scheme` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`an unworkable regulatory scheme` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `an unworkable regulatory scheme` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `an unworkable regulatory scheme` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. An unworkable regulatory scheme may look strict but fail in practice. 译：一套不可操作的监管方案看起来严格，但在实践中可能失败。&lt;br&gt;2. An unworkable regulatory scheme can reshape decisions made by governments, firms and families. 译：an unworkable regulatory scheme 会重塑政府、企业和家庭作出的决定。&lt;br&gt;3. Public policy should respond to an unworkable regulatory scheme before it becomes a larger social problem. 译：公共政策应当在 an unworkable regulatory scheme 变成更大的社会问题之前作出回应。
 &lt;b&gt;其他可用地方&lt;/b&gt;：政策评估、科技治理、作文批判。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：unworkable
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：行不通的；不可操作的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：workable 不是“能工作的”，而是“可执行/可操作”。 例：The expression `an unworkable regulatory scheme` should be interpreted through its context. 译：表达 `an unworkable regulatory scheme` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：an unworkable regulatory scheme；本卡覆盖这些变体：unworkable
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：行不通的；不可操作的。例：An unworkable regulatory scheme may look strict but fail in practice. 译：一套不可操作的监管方案看起来严格，但在实践中可能失败。 2. 文章义/考试义：workable 不是“能工作的”，而是“可执行/可操作”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：An unworkable regulatory scheme may look strict but fail in practice. 译：一套不可操作的监管方案看起来严格，但在实践中可能失败。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：An unworkable regulatory scheme can reshape decisions made by governments, firms and families. 译：an unworkable regulatory scheme 会重塑政府、企业和家庭作出的决定。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -520,7 +507,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：便宜且可塑/易改造的
 &lt;b&gt;考研核心考点&lt;/b&gt;：双形容词并列，描述技术扩散条件
-&lt;b&gt;词汇拆解&lt;/b&gt;：cheap = 成本低；malleable = 易被改变/改造｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：cheap = 成本低；malleable = 易被改变/改造。中文：这是一个名词短语，本卡重点是把 `cheap and malleable AI models` 和“便宜且可塑/易改造的”一起记，尤其注意搭配对象和语境义。English: `cheap and malleable AI models` functions as a noun phrase; learn the whole chunk with its meaning `便宜且可塑/易改造的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：cheap 不总是贬义，可指低成本；malleable 可褒可贬。
 &lt;b&gt;语气色彩&lt;/b&gt;：中性中带风险。</t>
         </is>
@@ -532,13 +519,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：推理题可能问为什么难以控制。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到并列形容词，注意共同服务于后面的名词。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：low-cost and adaptable; inexpensive and easy to modify
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Cheap and malleable AI models can support innovation and misuse at the same time. 译：便宜且可塑的人工智能模型既能支持创新，也可能支持滥用。&lt;br&gt;2. In an exam passage, `cheap and malleable AI models` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`cheap and malleable AI models` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `cheap and malleable AI models` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `cheap and malleable AI models` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Cheap and malleable AI models can support innovation and misuse at the same time. 译：便宜且可塑的人工智能模型既能支持创新，也可能支持滥用。&lt;br&gt;2. Clear public rules can make cheap and malleable AI models safer and more accountable. 译：清晰的公共规则可以让 cheap and malleable AI models 更安全、更可问责。&lt;br&gt;3. Without social responsibility, cheap and malleable AI models may create risks that spread beyond one company. 译：如果缺乏社会责任，cheap and malleable AI models 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、教育工具、创新风险。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：malleable；cheap and malleable
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：便宜且可塑/易改造的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：cheap 不总是贬义，可指低成本；malleable 可褒可贬。 例：The expression `cheap and malleable AI models` should be interpreted through its context. 译：表达 `cheap and malleable AI models` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：cheap and malleable AI models；本卡覆盖这些变体：malleable；cheap and malleable
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：便宜且可塑/易改造的。例：Cheap and malleable AI models can support innovation and misuse at the same time. 译：便宜且可塑的人工智能模型既能支持创新，也可能支持滥用。 2. 文章义/考试义：cheap 不总是贬义，可指低成本；malleable 可褒可贬。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Cheap and malleable AI models can support innovation and misuse at the same time. 译：便宜且可塑的人工智能模型既能支持创新，也可能支持滥用。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make cheap and malleable AI models safer and more accountable. 译：清晰的公共规则可以让 cheap and malleable AI models 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -557,7 +543,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：公开可用模型与受限模型之间的巨大差距是个问题
 &lt;b&gt;考研核心考点&lt;/b&gt;：抽象主语 + 系表结构
-&lt;b&gt;词汇拆解&lt;/b&gt;：publicly available = 公开可得；restricted = 受限制的；gulf = 巨大差距｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：publicly available = 公开可得；restricted = 受限制的；gulf = 巨大差距。中文：这是一个名词短语，本卡重点是把 `a gulf between publicly available and restricted models` 和“公开可用模型与受限模型之间的巨大差距是个问题”一起记，尤其注意搭配对象和语境义。English: `a gulf between publicly available and restricted models` functions as a noun phrase; learn the whole chunk with its meaning `公开可用模型与受限模型之间的巨大差距是个问题` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：available 是“可获得的”，不是“有空的”；restricted 是“受限的”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、问题判断。</t>
         </is>
@@ -569,13 +555,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题考多重前置修饰和 A-B 对比。
 &lt;b&gt;答题技巧&lt;/b&gt;：先抓主干：a gulf is a problem；中间是 between 短语。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：a divide between open and closed systems; a gap between public and restricted access
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A gulf between publicly available and restricted models could create a sudden shock. 译：公开可用模型与受限模型之间的巨大差距可能造成突然冲击。&lt;br&gt;2. In an exam passage, `a gulf between publicly available and restricted models` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`a gulf between publicly available and restricted models` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `a gulf between publicly available and restricted models` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `a gulf between publicly available and restricted models` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A gulf between publicly available and restricted models could create a sudden shock. 译：公开可用模型与受限模型之间的巨大差距可能造成突然冲击。&lt;br&gt;2. A gulf between publicly available and restricted models can reshape decisions made by governments, firms and families. 译：a gulf between publicly available and restricted models 会重塑政府、企业和家庭作出的决定。&lt;br&gt;3. Public policy should respond to a gulf between publicly available and restricted models before it becomes a larger social problem. 译：公共政策应当在 a gulf between publicly available and restricted models 变成更大的社会问题之前作出回应。
 &lt;b&gt;其他可用地方&lt;/b&gt;：教育公平、科技鸿沟、社会责任。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：a gulf between A and B；a gulf between publicly available and restricted models is a problem.
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：公开可用模型与受限模型之间的巨大差距是个问题。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：available 是“可获得的”，不是“有空的”；restricted 是“受限的”。 例：The expression `a gulf between publicly available and restricted models` should be interpreted through its context. 译：表达 `a gulf between publicly available and restricted models` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：a gulf between publicly available and restricted models；本卡覆盖这些变体：a gulf between A and B；a gulf between publicly available and restricted models is a problem.
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：公开可用模型与受限模型之间的巨大差距是个问题。例：A gulf between publicly available and restricted models could create a sudden shock. 译：公开可用模型与受限模型之间的巨大差距可能造成突然冲击。 2. 文章义/考试义：available 是“可获得的”，不是“有空的”；restricted 是“受限的”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A gulf between publicly available and restricted models could create a sudden shock. 译：公开可用模型与受限模型之间的巨大差距可能造成突然冲击。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：A gulf between publicly available and restricted models can reshape decisions made by governments, firms and families. 译：a gulf between publicly available and restricted models 会重塑政府、企业和家庭作出的决定。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -594,7 +579,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：压住；封锁；憋住；限制流动
 &lt;b&gt;考研核心考点&lt;/b&gt;：短语动词，常用于情绪、信息、技术扩散
-&lt;b&gt;词汇拆解&lt;/b&gt;：bottle = 瓶子；bottle up = 把……装瓶里，引申为压住。｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：bottle = 瓶子；bottle up = 把……装瓶里，引申为压住。。中文：这是一个固定搭配或外刊表达，本卡重点是把 `bottle up powerful technology` 和“压住；封锁；憋住；限制流动”一起记，尤其注意搭配对象和语境义。English: `bottle up powerful technology` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `压住；封锁；憋住；限制流动` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：可指压抑情绪，也可指封锁资源/信息。
 &lt;b&gt;语气色彩&lt;/b&gt;：形象、略口语。</t>
         </is>
@@ -606,13 +591,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题会考非字面义。
 &lt;b&gt;答题技巧&lt;/b&gt;：对象若是 emotion/information/technology，译为“压抑/封锁/限制”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：hold back; contain; suppress; lock up
-&lt;b&gt;多场景例句&lt;/b&gt;：1. It is difficult to bottle up powerful technology once people know how useful it is. 译：一旦人们知道强大技术有多有用，就很难把它长期封锁起来。&lt;br&gt;2. In an exam passage, `bottle up powerful technology` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`bottle up powerful technology` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `bottle up powerful technology` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `bottle up powerful technology` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. It is difficult to bottle up powerful technology once people know how useful it is. 译：一旦人们知道强大技术有多有用，就很难把它长期封锁起来。&lt;br&gt;2. Clear public rules can make bottle up powerful technology safer and more accountable. 译：清晰的公共规则可以让 bottle up powerful technology 更安全、更可问责。&lt;br&gt;3. Without social responsibility, bottle up powerful technology may create risks that spread beyond one company. 译：如果缺乏社会责任，bottle up powerful technology 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技扩散、心理健康、社会治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：bottle up
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：压住；封锁；憋住；限制流动。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：可指压抑情绪，也可指封锁资源/信息。 例：The expression `bottle up powerful technology` should be interpreted through its context. 译：表达 `bottle up powerful technology` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：bottle up powerful technology；本卡覆盖这些变体：bottle up
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：压住；封锁；憋住；限制流动。例：It is difficult to bottle up powerful technology once people know how useful it is. 译：一旦人们知道强大技术有多有用，就很难把它长期封锁起来。 2. 文章义/考试义：可指压抑情绪，也可指封锁资源/信息。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：It is difficult to bottle up powerful technology once people know how useful it is. 译：一旦人们知道强大技术有多有用，就很难把它长期封锁起来。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make bottle up powerful technology safer and more accountable. 译：清晰的公共规则可以让 bottle up powerful technology 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -631,7 +615,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：分阶段发布；错峰释放
 &lt;b&gt;考研核心考点&lt;/b&gt;：科技产品/政策执行类实用搭配
-&lt;b&gt;词汇拆解&lt;/b&gt;：staggered = 分阶段的/错开的；release = 发布/释放｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：staggered = 分阶段的/错开的；release = 发布/释放。中文：这是一个固定搭配或外刊表达，本卡重点是把 `staggered release` 和“分阶段发布；错峰释放”一起记，尤其注意搭配对象和语境义。English: `staggered release` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `分阶段发布；错峰释放` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：release 不只是“释放犯人”，也指产品发布、模型开放。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性。</t>
         </is>
@@ -643,12 +627,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会把 staggered 替换为 phased/gradual。
 &lt;b&gt;答题技巧&lt;/b&gt;：翻译为“分阶段发布”，不要译成“蹒跚发布”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：phased release; gradual rollout; controlled release
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A staggered release may reduce the shock caused by a powerful new technology. 译：分阶段发布可能减少强大新技术造成的冲击。&lt;br&gt;2. In an exam passage, `staggered release` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`staggered release` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `staggered release` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `staggered release` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A staggered release may reduce the shock caused by a powerful new technology. 译：分阶段发布可能减少强大新技术造成的冲击。&lt;br&gt;2. Public institutions should consider how staggered release affects fairness, efficiency and trust. 译：公共机构应考虑 staggered release 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss staggered release without ignoring long-term responsibility. 译：一个成熟社会可以讨论 staggered release，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技治理、产品发布、政策改革。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：分阶段发布；错峰释放。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：release 不只是“释放犯人”，也指产品发布、模型开放。 例：The expression `staggered release` should be interpreted through its context. 译：表达 `staggered release` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：staggered release
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：分阶段发布；错峰释放。例：A staggered release may reduce the shock caused by a powerful new technology. 译：分阶段发布可能减少强大新技术造成的冲击。 2. 文章义/考试义：release 不只是“释放犯人”，也指产品发布、模型开放。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A staggered release may reduce the shock caused by a powerful new technology. 译：分阶段发布可能减少强大新技术造成的冲击。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how staggered release affects fairness, efficiency and trust. 译：公共机构应考虑 staggered release 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -667,7 +650,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：使正式化；把……制度化
 &lt;b&gt;考研核心考点&lt;/b&gt;：制度建设高频动词
-&lt;b&gt;词汇拆解&lt;/b&gt;：formal = 正式的；-ise = 使……化｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：formal = 正式的；-ise = 使……化。中文：这是一个固定搭配或外刊表达，本卡重点是把 `formalise safety rules` 和“使正式化；把……制度化”一起记，尤其注意搭配对象和语境义。English: `formalise safety rules` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `使正式化；把……制度化` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不是“形式化”那么空，可译为“确立正式制度”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性偏政策。</t>
         </is>
@@ -679,13 +662,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：写作中可用于制度、标准、程序。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 formalise + arrangement/rules/process，译为“将……制度化”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：institutionalise; codify; make official
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Governments should formalise safety rules instead of relying on informal promises. 译：政府应当把安全规则正式化，而不是依赖非正式承诺。&lt;br&gt;2. In an exam passage, `formalise safety rules` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`formalise safety rules` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `formalise safety rules` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `formalise safety rules` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Governments should formalise safety rules instead of relying on informal promises. 译：政府应当把安全规则正式化，而不是依赖非正式承诺。&lt;br&gt;2. Clear public rules can make formalise safety rules safer and more accountable. 译：清晰的公共规则可以让 formalise safety rules 更安全、更可问责。&lt;br&gt;3. Without social responsibility, formalise safety rules may create risks that spread beyond one company. 译：如果缺乏社会责任，formalise safety rules 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：制度建设、职场流程、科技监管。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：formalise；formalising
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：使正式化；把……制度化。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：不是“形式化”那么空，可译为“确立正式制度”。 例：The expression `formalise safety rules` should be interpreted through its context. 译：表达 `formalise safety rules` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：formalise safety rules；本卡覆盖这些变体：formalise；formalising
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：使正式化；把……制度化。例：Governments should formalise safety rules instead of relying on informal promises. 译：政府应当把安全规则正式化，而不是依赖非正式承诺。 2. 文章义/考试义：不是“形式化”那么空，可译为“确立正式制度”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Governments should formalise safety rules instead of relying on informal promises. 译：政府应当把安全规则正式化，而不是依赖非正式承诺。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make formalise safety rules safer and more accountable. 译：清晰的公共规则可以让 formalise safety rules 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -704,7 +686,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：事无巨细地管理；过度干预
 &lt;b&gt;考研核心考点&lt;/b&gt;：管理类负面词
-&lt;b&gt;词汇拆解&lt;/b&gt;：micro = 微小；manage = 管理｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：micro = 微小；manage = 管理。中文：这是一个固定搭配或外刊表达，本卡重点是把 `micromanage` 和“事无巨细地管理；过度干预”一起记，尤其注意搭配对象和语境义。English: `micromanage` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `事无巨细地管理；过度干预` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不是普通 manage，而是管得过细。
 &lt;b&gt;语气色彩&lt;/b&gt;：批评性。</t>
         </is>
@@ -716,12 +698,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题负面；常与 bureaucracy 搭配。
 &lt;b&gt;答题技巧&lt;/b&gt;：译为“过度干预/微观管理”，不要只译“管理”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：overmanage; interfere in details; regulate every detail
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators should set clear goals, but they should not micromanage every technical detail. 译：监管者应当设定明确目标，但不应事无巨细地管理每个技术细节。&lt;br&gt;2. In an exam passage, `micromanage` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`micromanage` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `micromanage` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `micromanage` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators should set clear goals, but they should not micromanage every technical detail. 译：监管者应当设定明确目标，但不应事无巨细地管理每个技术细节。&lt;br&gt;2. Public institutions should consider how micromanage affects fairness, efficiency and trust. 译：公共机构应考虑 micromanage 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss micromanage without ignoring long-term responsibility. 译：一个成熟社会可以讨论 micromanage，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：职场管理、教育管理、政府监管。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：事无巨细地管理；过度干预。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：不是普通 manage，而是管得过细。 例：The expression `micromanage` should be interpreted through its context. 译：表达 `micromanage` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：micromanage
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：事无巨细地管理；过度干预。例：Regulators should set clear goals, but they should not micromanage every technical detail. 译：监管者应当设定明确目标，但不应事无巨细地管理每个技术细节。 2. 文章义/考试义：不是普通 manage，而是管得过细。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Regulators should set clear goals, but they should not micromanage every technical detail. 译：监管者应当设定明确目标，但不应事无巨细地管理每个技术细节。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how micromanage affects fairness, efficiency and trust. 译：公共机构应考虑 micromanage 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -740,7 +721,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：与 AI 公司讨价还价/利益交换
 &lt;b&gt;考研核心考点&lt;/b&gt;：具体化的政治经济搭配
-&lt;b&gt;词汇拆解&lt;/b&gt;：horse-trading = 幕后交易/讨价还价；with AI companies = 对象｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：horse-trading = 幕后交易/讨价还价；with AI companies = 对象。中文：这是一个名词短语，本卡重点是把 `horse-trade with AI companies` 和“与 AI 公司讨价还价/利益交换”一起记，尤其注意搭配对象和语境义。English: `horse-trade with AI companies` functions as a noun phrase; learn the whole chunk with its meaning `与 AI 公司讨价还价/利益交换` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：horse-trading 比 negotiation 更带利益交换味。
 &lt;b&gt;语气色彩&lt;/b&gt;：新闻批评语气。</t>
         </is>
@@ -752,13 +733,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：推理题可考 regulatory capture。
 &lt;b&gt;答题技巧&lt;/b&gt;：译出“讨价还价/利益交换”，不要中性化成“合作”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：bargaining with firms; cutting deals with companies; regulatory horse-trading
-&lt;b&gt;多场景例句&lt;/b&gt;：1. The public may lose trust if regulators horse-trade with AI companies behind closed doors. 译：如果监管者与人工智能公司幕后讨价还价，公众可能会失去信任。&lt;br&gt;2. In an exam passage, `horse-trade with AI companies` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`horse-trade with AI companies` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `horse-trade with AI companies` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `horse-trade with AI companies` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. The public may lose trust if regulators horse-trade with AI companies behind closed doors. 译：如果监管者与人工智能公司幕后讨价还价，公众可能会失去信任。&lt;br&gt;2. Clear public rules can make horse-trade with AI companies safer and more accountable. 译：清晰的公共规则可以让 horse-trade with AI companies 更安全、更可问责。&lt;br&gt;3. Without social responsibility, horse-trade with AI companies may create risks that spread beyond one company. 译：如果缺乏社会责任，horse-trade with AI companies 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：企业责任、科技监管、公共伦理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：horse-trade；horse-trading with AI companies
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：与 AI 公司讨价还价/利益交换。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：horse-trading 比 negotiation 更带利益交换味。 例：The expression `horse-trade with AI companies` should be interpreted through its context. 译：表达 `horse-trade with AI companies` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：horse-trade with AI companies；本卡覆盖这些变体：horse-trade；horse-trading with AI companies
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：与 AI 公司讨价还价/利益交换。例：The public may lose trust if regulators horse-trade with AI companies behind closed doors. 译：如果监管者与人工智能公司幕后讨价还价，公众可能会失去信任。 2. 文章义/考试义：horse-trading 比 negotiation 更带利益交换味。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：The public may lose trust if regulators horse-trade with AI companies behind closed doors. 译：如果监管者与人工智能公司幕后讨价还价，公众可能会失去信任。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make horse-trade with AI companies safer and more accountable. 译：清晰的公共规则可以让 horse-trade with AI companies 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -777,7 +757,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：退后观察；暂不干预
 &lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语：stand 不只是站立
-&lt;b&gt;词汇拆解&lt;/b&gt;：stand back = move away / refrain from intervening｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：stand back = move away / refrain from intervening。中文：这是一个固定搭配或外刊表达，本卡重点是把 `stand back` 和“退后观察；暂不干预”一起记，尤其注意搭配对象和语境义。English: `stand back` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `退后观察；暂不干预` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：可指身体退后，也可指政策上不插手。
 &lt;b&gt;语气色彩&lt;/b&gt;：中性，政策语境中可能暗示克制。</t>
         </is>
@@ -789,12 +769,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题常考抽象义“旁观/不插手”。
 &lt;b&gt;答题技巧&lt;/b&gt;：结合对象判断：stand back from markets = 不干预市场。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：step back; refrain from intervening; take a broader view
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Sometimes policymakers should stand back and examine the whole system. 译：有时政策制定者应当退后一步，审视整个系统。&lt;br&gt;2. In an exam passage, `stand back` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`stand back` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `stand back` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `stand back` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Sometimes policymakers should stand back and examine the whole system. 译：有时政策制定者应当退后一步，审视整个系统。&lt;br&gt;2. Public institutions should consider how stand back affects fairness, efficiency and trust. 译：公共机构应考虑 stand back 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss stand back without ignoring long-term responsibility. 译：一个成熟社会可以讨论 stand back，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：职场管理、政策监管、个人决策。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：退后观察；暂不干预。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：可指身体退后，也可指政策上不插手。 例：The expression `stand back` should be interpreted through its context. 译：表达 `stand back` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：stand back
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：退后观察；暂不干预。例：Sometimes policymakers should stand back and examine the whole system. 译：有时政策制定者应当退后一步，审视整个系统。 2. 文章义/考试义：可指身体退后，也可指政策上不插手。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Sometimes policymakers should stand back and examine the whole system. 译：有时政策制定者应当退后一步，审视整个系统。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how stand back affects fairness, efficiency and trust. 译：公共机构应考虑 stand back 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -813,7 +792,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：合并；整合
 &lt;b&gt;考研核心考点&lt;/b&gt;：正式动词，常用于机构、规则、系统
-&lt;b&gt;词汇拆解&lt;/b&gt;：amalgam = 混合物；-ate 动词化｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：amalgam = 混合物；-ate 动词化。中文：这是一个可替换词组，本卡重点是把 `amalgamate rules/agencies` 和“合并；整合”一起记，尤其注意搭配对象和语境义。English: `amalgamate rules/agencies` functions as a interchangeable phrase pattern; learn the whole chunk with its meaning `合并；整合` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：比 combine 更正式，强调合成一个整体。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性。</t>
         </is>
@@ -825,13 +804,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中常与 agencies/data/rules 搭配。
 &lt;b&gt;答题技巧&lt;/b&gt;：选项 merge/integrate/consolidate 是同义替换。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：merge; integrate; consolidate; combine
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A country may need to amalgamate rules and agencies to regulate a complex industry. 译：一个国家可能需要整合规则和机构来监管复杂行业。&lt;br&gt;2. In an exam passage, `amalgamate rules/agencies` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`amalgamate rules/agencies` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `amalgamate rules/agencies` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `amalgamate rules/agencies` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A country may need to amalgamate rules and agencies to regulate a complex industry. 译：一个国家可能需要整合规则和机构来监管复杂行业。&lt;br&gt;2. Clear public rules can make amalgamate rules/agencies safer and more accountable. 译：清晰的公共规则可以让 amalgamate rules/agencies 更安全、更可问责。&lt;br&gt;3. Without social responsibility, amalgamate rules/agencies may create risks that spread beyond one company. 译：如果缺乏社会责任，amalgamate rules/agencies 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：制度建设、组织管理、科技治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：amalgamate
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：合并；整合。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：比 combine 更正式，强调合成一个整体。 例：The expression `amalgamate rules/agencies` should be interpreted through its context. 译：表达 `amalgamate rules/agencies` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：amalgamate rules/agencies；本卡覆盖这些变体：amalgamate
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：合并；整合。例：A country may need to amalgamate rules and agencies to regulate a complex industry. 译：一个国家可能需要整合规则和机构来监管复杂行业。 2. 文章义/考试义：比 combine 更正式，强调合成一个整体。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A country may need to amalgamate rules and agencies to regulate a complex industry. 译：一个国家可能需要整合规则和机构来监管复杂行业。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make amalgamate rules/agencies safer and more accountable. 译：清晰的公共规则可以让 amalgamate rules/agencies 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -850,7 +828,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：建立筹码；增强谈判/影响力
 &lt;b&gt;考研核心考点&lt;/b&gt;：政治经济类核心搭配
-&lt;b&gt;词汇拆解&lt;/b&gt;：leverage = 杠杆；引申为影响力/谈判筹码｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：leverage = 杠杆；引申为影响力/谈判筹码。中文：这是一个名词短语，本卡重点是把 `build leverage over AI companies` 和“建立筹码；增强谈判/影响力”一起记，尤其注意搭配对象和语境义。English: `build leverage over AI companies` functions as a noun phrase; learn the whole chunk with its meaning `建立筹码；增强谈判/影响力` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：leverage 不是普通“杠杆”，常指可利用的权力优势。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、策略色彩。</t>
         </is>
@@ -862,13 +840,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节/推理题常用 influence/bargaining power 替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：译为“建立筹码/增强制衡能力”更贴政策语境。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：gain leverage; increase bargaining power; strengthen influence
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators can build leverage over AI companies by developing technical expertise. 译：监管者可以通过发展技术专业能力来增强对人工智能公司的制衡能力。&lt;br&gt;2. In an exam passage, `build leverage over AI companies` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`build leverage over AI companies` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `build leverage over AI companies` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `build leverage over AI companies` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulators can build leverage over AI companies by developing technical expertise. 译：监管者可以通过发展技术专业能力来增强对人工智能公司的制衡能力。&lt;br&gt;2. Clear public rules can make build leverage over AI companies safer and more accountable. 译：清晰的公共规则可以让 build leverage over AI companies 更安全、更可问责。&lt;br&gt;3. Without social responsibility, build leverage over AI companies may create risks that spread beyond one company. 译：如果缺乏社会责任，build leverage over AI companies 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：职场谈判、国际关系、政府监管。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：build leverage
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：建立筹码；增强谈判/影响力。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：leverage 不是普通“杠杆”，常指可利用的权力优势。 例：The expression `build leverage over AI companies` should be interpreted through its context. 译：表达 `build leverage over AI companies` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：build leverage over AI companies；本卡覆盖这些变体：build leverage
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：建立筹码；增强谈判/影响力。例：Regulators can build leverage over AI companies by developing technical expertise. 译：监管者可以通过发展技术专业能力来增强对人工智能公司的制衡能力。 2. 文章义/考试义：leverage 不是普通“杠杆”，常指可利用的权力优势。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Regulators can build leverage over AI companies by developing technical expertise. 译：监管者可以通过发展技术专业能力来增强对人工智能公司的制衡能力。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make build leverage over AI companies safer and more accountable. 译：清晰的公共规则可以让 build leverage over AI companies 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -887,7 +864,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：故障保护机制；失效安全的
 &lt;b&gt;考研核心考点&lt;/b&gt;：安全工程和制度设计词
-&lt;b&gt;词汇拆解&lt;/b&gt;：fail = 失败；safe = 安全；合起来指失败时仍安全。｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：fail = 失败；safe = 安全；合起来指失败时仍安全。。中文：这是一个固定搭配或外刊表达，本卡重点是把 `build a fail-safe into policy` 和“故障保护机制；失效安全的”一起记，尤其注意搭配对象和语境义。English: `build a fail-safe into policy` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `故障保护机制；失效安全的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不是“失败是安全的”，而是“即使出故障也能保证安全”。可作名词或形容词。
 &lt;b&gt;语气色彩&lt;/b&gt;：技术正式语体。</t>
         </is>
@@ -899,13 +876,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题不要拆成“失败-安全”，译为“故障保护”。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 fail-safe，要想到“预案/保护底线”，不是普通 safety。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：safety backstop; emergency safeguard; backup protection
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A wise government should build a fail-safe into policy before a crisis begins. 译：明智的政府应当在危机开始前把故障保护机制纳入政策。&lt;br&gt;2. In an exam passage, `build a fail-safe into policy` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`build a fail-safe into policy` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `build a fail-safe into policy` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `build a fail-safe into policy` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A wise government should build a fail-safe into policy before a crisis begins. 译：明智的政府应当在危机开始前把故障保护机制纳入政策。&lt;br&gt;2. Clear public rules can make build a fail-safe into policy safer and more accountable. 译：清晰的公共规则可以让 build a fail-safe into policy 更安全、更可问责。&lt;br&gt;3. Without social responsibility, build a fail-safe into policy may create risks that spread beyond one company. 译：如果缺乏社会责任，build a fail-safe into policy 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技安全、公共安全、风险管理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：fail-safe
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：故障保护机制；失效安全的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：不是“失败是安全的”，而是“即使出故障也能保证安全”。可作名词或形容词。 例：The expression `build a fail-safe into policy` should be interpreted through its context. 译：表达 `build a fail-safe into policy` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：build a fail-safe into policy；本卡覆盖这些变体：fail-safe
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：故障保护机制；失效安全的。例：A wise government should build a fail-safe into policy before a crisis begins. 译：明智的政府应当在危机开始前把故障保护机制纳入政策。 2. 文章义/考试义：不是“失败是安全的”，而是“即使出故障也能保证安全”。可作名词或形容词。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A wise government should build a fail-safe into policy before a crisis begins. 译：明智的政府应当在危机开始前把故障保护机制纳入政策。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make build a fail-safe into policy safer and more accountable. 译：清晰的公共规则可以让 build a fail-safe into policy 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -924,7 +900,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：灾难发生/降临
 &lt;b&gt;考研核心考点&lt;/b&gt;：新闻体灾难表达
-&lt;b&gt;词汇拆解&lt;/b&gt;：catastrophe = 大灾难；strike = 突然袭击/发生｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：catastrophe = 大灾难；strike = 突然袭击/发生。中文：这是一个句子/从句结构，本卡重点是把 `when catastrophe strikes` 和“灾难发生/降临”一起记，尤其注意搭配对象和语境义。English: `when catastrophe strikes` functions as a sentence or clause pattern; learn the whole chunk with its meaning `灾难发生/降临` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：strike 不只是“打击/罢工”，可指灾难突然发生。
 &lt;b&gt;语气色彩&lt;/b&gt;：强负面、新闻感。</t>
         </is>
@@ -936,13 +912,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义：strike = happen suddenly。
 &lt;b&gt;答题技巧&lt;/b&gt;：遇到 disaster/catastrophe + strike，译“发生/降临”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：disaster hits; crisis erupts; calamity occurs
-&lt;b&gt;多场景例句&lt;/b&gt;：1. When catastrophe strikes, improvised rules are often too late. 译：当灾难发生时，临时拼凑的规则往往已经太迟。&lt;br&gt;2. In an exam passage, `when catastrophe strikes` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`when catastrophe strikes` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `when catastrophe strikes` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `when catastrophe strikes` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. When catastrophe strikes, improvised rules are often too late. 译：当灾难发生时，临时拼凑的规则往往已经太迟。&lt;br&gt;2. When catastrophe strikes because capital, talent and policy often move together. 译：when catastrophe strikes，因为资本、人才和政策往往会共同移动。&lt;br&gt;3. Readers should notice how the sentence `when catastrophe strikes` links one change with another. 译：读者应注意 `when catastrophe strikes` 这个句子如何把一个变化与另一个变化连接起来。
 &lt;b&gt;其他可用地方&lt;/b&gt;：环境、健康、公共安全。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：catastrophe strikes
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：灾难发生/降临。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：strike 不只是“打击/罢工”，可指灾难突然发生。 例：The expression `when catastrophe strikes` should be interpreted through its context. 译：表达 `when catastrophe strikes` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：when catastrophe strikes；本卡覆盖这些变体：catastrophe strikes
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：灾难发生/降临。例：When catastrophe strikes, improvised rules are often too late. 译：当灾难发生时，临时拼凑的规则往往已经太迟。 2. 文章义/考试义：strike 不只是“打击/罢工”，可指灾难突然发生。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：When catastrophe strikes, improvised rules are often too late. 译：当灾难发生时，临时拼凑的规则往往已经太迟。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：When catastrophe strikes because capital, talent and policy often move together. 译：when catastrophe strikes，因为资本、人才和政策往往会共同移动。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -961,7 +936,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：被突然加上出口管制
 &lt;b&gt;考研核心考点&lt;/b&gt;：slap with = 突然强加处罚/限制
-&lt;b&gt;词汇拆解&lt;/b&gt;：slap = 拍打；slap A with B = 对 A 强加 B｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：slap = 拍打；slap A with B = 对 A 强加 B。中文：这是一个固定搭配或外刊表达，本卡重点是把 `slapped with export controls` 和“被突然加上出口管制”一起记，尤其注意搭配对象和语境义。English: `slapped with export controls` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `被突然加上出口管制` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：slap 熟词僻义：非身体动作，而是政策处罚。
 &lt;b&gt;语气色彩&lt;/b&gt;：新闻口吻，带突然和强硬感。</t>
         </is>
@@ -973,12 +948,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题会用 impose 替换 slapped with。
 &lt;b&gt;答题技巧&lt;/b&gt;：译为“被加征/被施加/被突然纳入管制”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：be hit with; be subject to; be placed under controls
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A company slapped with export controls may lose access to key markets. 译：一家被施加出口管制的公司可能会失去进入关键市场的机会。&lt;br&gt;2. In an exam passage, `slapped with export controls` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`slapped with export controls` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `slapped with export controls` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `slapped with export controls` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A company slapped with export controls may lose access to key markets. 译：一家被施加出口管制的公司可能会失去进入关键市场的机会。&lt;br&gt;2. Public institutions should consider how slapped with export controls affects fairness, efficiency and trust. 译：公共机构应考虑 slapped with export controls 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss slapped with export controls without ignoring long-term responsibility. 译：一个成熟社会可以讨论 slapped with export controls，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：国际贸易、科技竞争、政策风险。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：被突然加上出口管制。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：slap 熟词僻义：非身体动作，而是政策处罚。 例：The expression `slapped with export controls` should be interpreted through its context. 译：表达 `slapped with export controls` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：slapped with export controls
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：被突然加上出口管制。例：A company slapped with export controls may lose access to key markets. 译：一家被施加出口管制的公司可能会失去进入关键市场的机会。 2. 文章义/考试义：slap 熟词僻义：非身体动作，而是政策处罚。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A company slapped with export controls may lose access to key markets. 译：一家被施加出口管制的公司可能会失去进入关键市场的机会。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how slapped with export controls affects fairness, efficiency and trust. 译：公共机构应考虑 slapped with export controls 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -997,7 +971,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：对报复/怨恨的担忧被缓解了
 &lt;b&gt;考研核心考点&lt;/b&gt;：被动结构 + 抽象名词，考翻译
-&lt;b&gt;词汇拆解&lt;/b&gt;：fears = 担忧；grudge = 怨恨/积怨；allay = 缓解｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：fears = 担忧；grudge = 怨恨/积怨；allay = 缓解。中文：这是一个固定搭配或外刊表达，本卡重点是把 `fears of X were allayed` 和“对报复/怨恨的担忧被缓解了”一起记，尤其注意搭配对象和语境义。English: `fears of X were allayed` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `对报复/怨恨的担忧被缓解了` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：allay 专接 fear/concern/anxiety，表示减轻担忧。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、新闻语体。</t>
         </is>
@@ -1009,13 +983,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题重点是被动与抽象名词处理。
 &lt;b&gt;答题技巧&lt;/b&gt;：可译主动：“这缓解了人们对……的担忧”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：concerns were eased; fears were dispelled; anxieties were reduced
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Fears of unfair competition were allayed by clearer rules. 译：对不公平竞争的担忧被更清晰的规则缓解了。&lt;br&gt;2. In an exam passage, `fears of X were allayed` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`fears of X were allayed` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `fears of X were allayed` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `fears of X were allayed` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Fears of unfair competition were allayed by clearer rules. 译：对不公平竞争的担忧被更清晰的规则缓解了。&lt;br&gt;2. Public institutions should consider how fears of X were allayed affects fairness, efficiency and trust. 译：公共机构应考虑 fears of X were allayed 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss fears of X were allayed without ignoring long-term responsibility. 译：一个成熟社会可以讨论 fears of X were allayed，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：政治伦理、公共信任、社会责任。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：Fears of a grudge were allayed
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：对报复/怨恨的担忧被缓解了。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：allay 专接 fear/concern/anxiety，表示减轻担忧。 例：The expression `fears of X were allayed` should be interpreted through its context. 译：表达 `fears of X were allayed` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：fears of X were allayed；本卡覆盖这些变体：Fears of a grudge were allayed
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：对报复/怨恨的担忧被缓解了。例：Fears of unfair competition were allayed by clearer rules. 译：对不公平竞争的担忧被更清晰的规则缓解了。 2. 文章义/考试义：allay 专接 fear/concern/anxiety，表示减轻担忧。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Fears of unfair competition were allayed by clearer rules. 译：对不公平竞争的担忧被更清晰的规则缓解了。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how fears of X were allayed affects fairness, efficiency and trust. 译：公共机构应考虑 fears of X were allayed 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1034,7 +1007,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：事实上的禁令
 &lt;b&gt;考研核心考点&lt;/b&gt;：法律/政策高频：de facto = 实际上的
-&lt;b&gt;词汇拆解&lt;/b&gt;：de facto 来自拉丁语，反义 de jure = 法律上的。｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：de facto 来自拉丁语，反义 de jure = 法律上的。。中文：这是一个固定搭配或外刊表达，本卡重点是把 `de facto ban` 和“事实上的禁令”一起记，尤其注意搭配对象和语境义。English: `de facto ban` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `事实上的禁令` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：表示形式上未禁止，效果上等于禁止。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、法律政治语体。</t>
         </is>
@@ -1046,12 +1019,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：推理题会考“实际影响”而非字面政策名称。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 de facto，选项里 in effect/in practice 常是替换。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：in effect; in practice; practical ban
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A policy may become a de facto ban even if it does not use the word 'ban'. 译：一项政策即使没有使用“禁令”一词，也可能成为事实上的禁令。&lt;br&gt;2. In an exam passage, `de facto ban` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`de facto ban` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `de facto ban` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `de facto ban` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A policy may become a de facto ban even if it does not use the word 'ban'. 译：一项政策即使没有使用“禁令”一词，也可能成为事实上的禁令。&lt;br&gt;2. Public institutions should consider how de facto ban affects fairness, efficiency and trust. 译：公共机构应考虑 de facto ban 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss de facto ban without ignoring long-term responsibility. 译：一个成熟社会可以讨论 de facto ban，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：政策分析、法律、国际贸易。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：事实上的禁令。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：表示形式上未禁止，效果上等于禁止。 例：The expression `de facto ban` should be interpreted through its context. 译：表达 `de facto ban` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：de facto ban
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：事实上的禁令。例：A policy may become a de facto ban even if it does not use the word 'ban'. 译：一项政策即使没有使用“禁令”一词，也可能成为事实上的禁令。 2. 文章义/考试义：表示形式上未禁止，效果上等于禁止。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A policy may become a de facto ban even if it does not use the word 'ban'. 译：一项政策即使没有使用“禁令”一词，也可能成为事实上的禁令。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how de facto ban affects fairness, efficiency and trust. 译：公共机构应考虑 de facto ban 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1070,7 +1042,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：在过去一个月的喧闹争议中
 &lt;b&gt;考研核心考点&lt;/b&gt;：brouhaha = 喧嚷/风波，外刊调侃词
-&lt;b&gt;词汇拆解&lt;/b&gt;：throughout = 在……整个期间；brouhaha = noisy fuss/controversy｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：throughout = 在……整个期间；brouhaha = noisy fuss/controversy。中文：这是一个固定搭配或外刊表达，本卡重点是把 `amid a political brouhaha` 和“在过去一个月的喧闹争议中”一起记，尤其注意搭配对象和语境义。English: `amid a political brouhaha` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `在过去一个月的喧闹争议中` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：brouhaha 不是严肃 crisis，而是媒体吵闹和政治喧嚣。
 &lt;b&gt;语气色彩&lt;/b&gt;：讽刺、轻微幽默。</t>
         </is>
@@ -1082,13 +1054,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中显示作者略带不耐烦或嘲讽。
 &lt;b&gt;答题技巧&lt;/b&gt;：可译“风波/喧嚣/一片吵嚷”，不要译“布鲁哈哈”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：uproar; fuss; noisy controversy; commotion
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Amid a political brouhaha, serious policy questions are often ignored. 译：在政治喧嚣中，严肃的政策问题常常被忽视。&lt;br&gt;2. In an exam passage, `amid a political brouhaha` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`amid a political brouhaha` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `amid a political brouhaha` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `amid a political brouhaha` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Amid a political brouhaha, serious policy questions are often ignored. 译：在政治喧嚣中，严肃的政策问题常常被忽视。&lt;br&gt;2. Public institutions should consider how amid a political brouhaha affects fairness, efficiency and trust. 译：公共机构应考虑 amid a political brouhaha 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss amid a political brouhaha without ignoring long-term responsibility. 译：一个成熟社会可以讨论 amid a political brouhaha，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：媒体舆论、政治争议、社会热点。
 &lt;b&gt;归一化合并&lt;/b&gt;：原表达 `throughout the past month's brouhaha` 已改为考研一可迁移原型 `amid a political brouhaha`。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：在过去一个月的喧闹争议中。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：brouhaha 不是严肃 crisis，而是媒体吵闹和政治喧嚣。 例：The expression `amid a political brouhaha` should be interpreted through its context. 译：表达 `amid a political brouhaha` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：amid a political brouhaha；原表达 `throughout the past month's brouhaha` 已改为考研一可迁移原型 `amid a political brouhaha`。
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：在过去一个月的喧闹争议中。例：Amid a political brouhaha, serious policy questions are often ignored. 译：在政治喧嚣中，严肃的政策问题常常被忽视。 2. 文章义/考试义：brouhaha 不是严肃 crisis，而是媒体吵闹和政治喧嚣。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Amid a political brouhaha, serious policy questions are often ignored. 译：在政治喧嚣中，严肃的政策问题常常被忽视。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how amid a political brouhaha affects fairness, efficiency and trust. 译：公共机构应考虑 amid a political brouhaha 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1107,7 +1078,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：但那最多只能争取几个月，或一年时间
 &lt;b&gt;考研核心考点&lt;/b&gt;：buy time = 争取时间，熟词僻义
-&lt;b&gt;词汇拆解&lt;/b&gt;：buy = 买；buy time = gain time；at most = 最多｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：buy = 买；buy time = gain time；at most = 最多。中文：这是一个固定搭配或外刊表达，本卡重点是把 `buy months, or a year at most` 和“但那最多只能争取几个月，或一年时间”一起记，尤其注意搭配对象和语境义。English: `buy months, or a year at most` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `但那最多只能争取几个月，或一年时间` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：buy 不一定是购买，可指换来/争取。
 &lt;b&gt;语气色彩&lt;/b&gt;：转折、现实主义语气。</t>
         </is>
@@ -1119,13 +1090,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题考 buy 的抽象义和 at most。
 &lt;b&gt;答题技巧&lt;/b&gt;：that 指前文措施；不要译为“买几个月”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：gain time; buy a little time; delay the problem temporarily
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A temporary measure may buy months, or a year at most. 译：一项临时措施可能最多争取几个月，或一年时间。&lt;br&gt;2. In an exam passage, `buy months, or a year at most` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`buy months, or a year at most` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `buy months, or a year at most` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `buy months, or a year at most` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A temporary measure may buy months, or a year at most. 译：一项临时措施可能最多争取几个月，或一年时间。&lt;br&gt;2. Public institutions should consider how buy months, or a year at most affects fairness, efficiency and trust. 译：公共机构应考虑 buy months, or a year at most 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss buy months, or a year at most without ignoring long-term responsibility. 译：一个成熟社会可以讨论 buy months, or a year at most，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：政策改革、时间管理、危机应对。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：But that buys months, or a year at most
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：但那最多只能争取几个月，或一年时间。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：buy 不一定是购买，可指换来/争取。 例：The expression `buy months, or a year at most` should be interpreted through its context. 译：表达 `buy months, or a year at most` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：buy months, or a year at most；本卡覆盖这些变体：But that buys months, or a year at most
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：但那最多只能争取几个月，或一年时间。例：A temporary measure may buy months, or a year at most. 译：一项临时措施可能最多争取几个月，或一年时间。 2. 文章义/考试义：buy 不一定是购买，可指换来/争取。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A temporary measure may buy months, or a year at most. 译：一项临时措施可能最多争取几个月，或一年时间。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how buy months, or a year at most affects fairness, efficiency and trust. 译：公共机构应考虑 buy months, or a year at most 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1144,7 +1114,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：不受欢迎的；不合意的；有害的
 &lt;b&gt;考研核心考点&lt;/b&gt;：态度评价词，正式负面
-&lt;b&gt;词汇拆解&lt;/b&gt;：un- = not；desirable = 值得拥有的/理想的｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：un- = not；desirable = 值得拥有的/理想的。中文：这是一个固定搭配或外刊表达，本卡重点是把 `undesirable` 和“不受欢迎的；不合意的；有害的”一起记，尤其注意搭配对象和语境义。English: `undesirable` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `不受欢迎的；不合意的；有害的` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：desirable 不只是“性感的”，在正式语境中是“可取的”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、负面但克制。</t>
         </is>
@@ -1156,12 +1126,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中是 mild negative。
 &lt;b&gt;答题技巧&lt;/b&gt;：选项 harmful/unwelcome/problematic 可替换。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：unwelcome; harmful; problematic; not ideal
-&lt;b&gt;多场景例句&lt;/b&gt;：1. An undesirable outcome should be prevented before it becomes irreversible. 译：不合意的结果应当在变得不可逆之前被阻止。&lt;br&gt;2. In an exam passage, `undesirable` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`undesirable` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `undesirable` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `undesirable` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. An undesirable outcome should be prevented before it becomes irreversible. 译：不合意的结果应当在变得不可逆之前被阻止。&lt;br&gt;2. Public institutions should consider how undesirable affects fairness, efficiency and trust. 译：公共机构应考虑 undesirable 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss undesirable without ignoring long-term responsibility. 译：一个成熟社会可以讨论 undesirable，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技伦理、健康饮食、社会责任。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：不受欢迎的；不合意的；有害的。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：desirable 不只是“性感的”，在正式语境中是“可取的”。 例：The expression `undesirable` should be interpreted through its context. 译：表达 `undesirable` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：undesirable
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：不受欢迎的；不合意的；有害的。例：An undesirable outcome should be prevented before it becomes irreversible. 译：不合意的结果应当在变得不可逆之前被阻止。 2. 文章义/考试义：desirable 不只是“性感的”，在正式语境中是“可取的”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：An undesirable outcome should be prevented before it becomes irreversible. 译：不合意的结果应当在变得不可逆之前被阻止。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how undesirable affects fairness, efficiency and trust. 译：公共机构应考虑 undesirable 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1180,7 +1149,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：极大地；非常
 &lt;b&gt;考研核心考点&lt;/b&gt;：强调副词，用于增强程度
-&lt;b&gt;词汇拆解&lt;/b&gt;：tremendous = 巨大的；-ly 副词｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：tremendous = 巨大的；-ly 副词。中文：这是一个可替换词组，本卡重点是把 `improve/increase tremendously` 和“极大地；非常”一起记，尤其注意搭配对象和语境义。English: `improve/increase tremendously` functions as a interchangeable phrase pattern; learn the whole chunk with its meaning `极大地；非常` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：比 very 更正式、更强。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、中性。</t>
         </is>
@@ -1192,13 +1161,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：完形/阅读中可能用 greatly/substantially 替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：写作可替换 very much，但别滥用。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：greatly; enormously; substantially; immensely
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Digital tools can improve learning tremendously when they are used wisely. 译：如果使用得当，数字工具能够极大改善学习。&lt;br&gt;2. In an exam passage, `improve/increase tremendously` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`improve/increase tremendously` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `improve/increase tremendously` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `improve/increase tremendously` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Digital tools can improve learning tremendously when they are used wisely. 译：如果使用得当，数字工具能够极大改善学习。&lt;br&gt;2. Public institutions should consider how improve/increase tremendously affects fairness, efficiency and trust. 译：公共机构应考虑 improve/increase tremendously 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss improve/increase tremendously without ignoring long-term responsibility. 译：一个成熟社会可以讨论 improve/increase tremendously，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：作文：教育进步、科技影响、健康改善。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：tremendously
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：极大地；非常。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：比 very 更正式、更强。 例：The expression `improve/increase tremendously` should be interpreted through its context. 译：表达 `improve/increase tremendously` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：improve/increase tremendously；本卡覆盖这些变体：tremendously
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：极大地；非常。例：Digital tools can improve learning tremendously when they are used wisely. 译：如果使用得当，数字工具能够极大改善学习。 2. 文章义/考试义：比 very 更正式、更强。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Digital tools can improve learning tremendously when they are used wisely. 译：如果使用得当，数字工具能够极大改善学习。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how improve/increase tremendously affects fairness, efficiency and trust. 译：公共机构应考虑 improve/increase tremendously 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1217,7 +1185,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：撇开对中国的担忧不谈
 &lt;b&gt;考研核心考点&lt;/b&gt;：让步/话题转移句首结构
-&lt;b&gt;词汇拆解&lt;/b&gt;：aside = 放在一边；A aside = leaving A aside｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：aside = 放在一边；A aside = leaving A aside。中文：这是一个固定搭配或外刊表达，本卡重点是把 `worries about X aside` 和“撇开对中国的担忧不谈”一起记，尤其注意搭配对象和语境义。English: `worries about X aside` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `撇开对中国的担忧不谈` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：aside 不只是“在旁边”，可表示暂且不谈。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、转折引导。</t>
         </is>
@@ -1229,13 +1197,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：长难句中常作句首状语，容易误判主干。
 &lt;b&gt;答题技巧&lt;/b&gt;：先把 aside 结构括起来，再找主句。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：leaving China aside; apart from concerns about China; setting aside geopolitical worries
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Worries about cost aside, the reform has clear educational value. 译：撇开成本方面的担忧不谈，这项改革具有明确的教育价值。&lt;br&gt;2. In an exam passage, `worries about X aside` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`worries about X aside` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `worries about X aside` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `worries about X aside` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Worries about cost aside, the reform has clear educational value. 译：撇开成本方面的担忧不谈，这项改革具有明确的教育价值。&lt;br&gt;2. Public institutions should consider how worries about X aside affects fairness, efficiency and trust. 译：公共机构应考虑 worries about X aside 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss worries about X aside without ignoring long-term responsibility. 译：一个成熟社会可以讨论 worries about X aside，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：议论文让步、科技伦理、国际关系。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：Worries about China aside
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：撇开对中国的担忧不谈。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：aside 不只是“在旁边”，可表示暂且不谈。 例：The expression `worries about X aside` should be interpreted through its context. 译：表达 `worries about X aside` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：worries about X aside；本卡覆盖这些变体：Worries about China aside
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：撇开对中国的担忧不谈。例：Worries about cost aside, the reform has clear educational value. 译：撇开成本方面的担忧不谈，这项改革具有明确的教育价值。 2. 文章义/考试义：aside 不只是“在旁边”，可表示暂且不谈。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Worries about cost aside, the reform has clear educational value. 译：撇开成本方面的担忧不谈，这项改革具有明确的教育价值。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how worries about X aside affects fairness, efficiency and trust. 译：公共机构应考虑 worries about X aside 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1254,7 +1221,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：一次巨大的猛然跃升/剧烈摇摆
 &lt;b&gt;考研核心考点&lt;/b&gt;：lurch = 突然倾斜/猛变，形象词
-&lt;b&gt;词汇拆解&lt;/b&gt;：great = 大的；lurch = sudden uncontrolled movement/change｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：great = 大的；lurch = sudden uncontrolled movement/change。中文：这是一个名词短语，本卡重点是把 `a great lurch in capability` 和“一次巨大的猛然跃升/剧烈摇摆”一起记，尤其注意搭配对象和语境义。English: `a great lurch in capability` functions as a noun phrase; learn the whole chunk with its meaning `一次巨大的猛然跃升/剧烈摇摆` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：lurch 可指身体踉跄，也可指政策/技术突然变化。
 &lt;b&gt;语气色彩&lt;/b&gt;：形象、负面，强调失控感。</t>
         </is>
@@ -1266,13 +1233,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题中 sudden shift/jump 可能替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：不要译成“伟大的倾斜”，译为“剧烈跃迁/突然摇摆”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：sudden jump; abrupt shift; uncontrolled swing
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A great lurch in capability can shock markets and regulators. 译：能力的剧烈跃升可能冲击市场和监管者。&lt;br&gt;2. In an exam passage, `a great lurch in capability` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`a great lurch in capability` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `a great lurch in capability` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `a great lurch in capability` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A great lurch in capability can shock markets and regulators. 译：能力的剧烈跃升可能冲击市场和监管者。&lt;br&gt;2. A great lurch in capability can reshape decisions made by governments, firms and families. 译：a great lurch in capability 会重塑政府、企业和家庭作出的决定。&lt;br&gt;3. Public policy should respond to a great lurch in capability before it becomes a larger social problem. 译：公共政策应当在 a great lurch in capability 变成更大的社会问题之前作出回应。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技变化、经济波动、政策转向。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：a great lurch
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：一次巨大的猛然跃升/剧烈摇摆。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：lurch 可指身体踉跄，也可指政策/技术突然变化。 例：The expression `a great lurch in capability` should be interpreted through its context. 译：表达 `a great lurch in capability` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：a great lurch in capability；本卡覆盖这些变体：a great lurch
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：一次巨大的猛然跃升/剧烈摇摆。例：A great lurch in capability can shock markets and regulators. 译：能力的剧烈跃升可能冲击市场和监管者。 2. 文章义/考试义：lurch 可指身体踉跄，也可指政策/技术突然变化。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A great lurch in capability can shock markets and regulators. 译：能力的剧烈跃升可能冲击市场和监管者。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：A great lurch in capability can reshape decisions made by governments, firms and families. 译：a great lurch in capability 会重塑政府、企业和家庭作出的决定。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1291,7 +1257,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：每当这些模型最终发布时，能力的突然跃升都会释放混乱
 &lt;b&gt;考研核心考点&lt;/b&gt;：时间状语从句 + 强调 did + would 预测后果
-&lt;b&gt;词汇拆解&lt;/b&gt;：sudden jump = 突然跃升；capability = 能力；unleash = 释放/引发；chaos = 混乱｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：sudden jump = 突然跃升；capability = 能力；unleash = 释放/引发；chaos = 混乱。中文：这是一个名词短语，本卡重点是把 `a sudden jump in capability would unleash chaos` 和“每当这些模型最终发布时，能力的突然跃升都会释放混乱”一起记，尤其注意搭配对象和语境义。English: `a sudden jump in capability would unleash chaos` functions as a noun phrase; learn the whole chunk with its meaning `每当这些模型最终发布时，能力的突然跃升都会释放混乱` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：did get released 中 did 强调“确实/最终会”。
 &lt;b&gt;语气色彩&lt;/b&gt;：强烈警告、负面预测。</t>
         </is>
@@ -1303,13 +1269,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：长难句考主干：jump would unleash chaos。
 &lt;b&gt;答题技巧&lt;/b&gt;：先删 whenever 从句；did 表强调，不译成“做发布”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：a sudden jump would unleash chaos; delayed release would cause disruption
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A sudden jump in capability would unleash chaos if society had no preparation. 译：如果社会毫无准备，能力的突然跃升会释放混乱。&lt;br&gt;2. In an exam passage, `a sudden jump in capability would unleash chaos` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`a sudden jump in capability would unleash chaos` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `a sudden jump in capability would unleash chaos` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `a sudden jump in capability would unleash chaos` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A sudden jump in capability would unleash chaos if society had no preparation. 译：如果社会毫无准备，能力的突然跃升会释放混乱。&lt;br&gt;2. A sudden jump in capability would unleash chaos can reshape decisions made by governments, firms and families. 译：a sudden jump in capability would unleash chaos 会重塑政府、企业和家庭作出的决定。&lt;br&gt;3. Public policy should respond to a sudden jump in capability would unleash chaos before it becomes a larger social problem. 译：公共政策应当在 a sudden jump in capability would unleash chaos 变成更大的社会问题之前作出回应。
 &lt;b&gt;其他可用地方&lt;/b&gt;：科技治理、经济风险、社会稳定。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：The sudden jump in capability whenever the models did get released would unleash chaos.
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：每当这些模型最终发布时，能力的突然跃升都会释放混乱。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：did get released 中 did 强调“确实/最终会”。 例：The expression `a sudden jump in capability would unleash chaos` should be interpreted through its context. 译：表达 `a sudden jump in capability would unleash chaos` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：a sudden jump in capability would unleash chaos；本卡覆盖这些变体：The sudden jump in capability whenever the models did get released would unleash chaos.
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：每当这些模型最终发布时，能力的突然跃升都会释放混乱。例：A sudden jump in capability would unleash chaos if society had no preparation. 译：如果社会毫无准备，能力的突然跃升会释放混乱。 2. 文章义/考试义：did get released 中 did 强调“确实/最终会”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A sudden jump in capability would unleash chaos if society had no preparation. 译：如果社会毫无准备，能力的突然跃升会释放混乱。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：A sudden jump in capability would unleash chaos can reshape decisions made by governments, firms and families. 译：a sudden jump in capability would unleash chaos 会重塑政府、企业和家庭作出的决定。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1328,7 +1293,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：专业知识；专门能力
 &lt;b&gt;考研核心考点&lt;/b&gt;：抽象名词，考研高频
-&lt;b&gt;词汇拆解&lt;/b&gt;：expert = 专家；-ise/-ise? expertise 名词 = 专业能力｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：expert = 专家；-ise/-ise? expertise 名词 = 专业能力。中文：这是一个固定搭配或外刊表达，本卡重点是把 `build technical expertise` 和“专业知识；专门能力”一起记，尤其注意搭配对象和语境义。English: `build technical expertise` functions as a fixed collocation / journalistic expression; learn the whole chunk with its meaning `专业知识；专门能力` and its usual context.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不可数名词，常搭配 technical/legal/scientific expertise。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、正面。</t>
         </is>
@@ -1340,13 +1305,12 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：细节题常用 knowledge/competence 替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：不要加复数；译为“专业知识/专门能力”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：specialised knowledge; technical competence; professional know-how
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Public agencies must build technical expertise before they regulate new technology. 译：公共机构在监管新技术之前必须建立技术专业能力。&lt;br&gt;2. In an exam passage, `build technical expertise` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`build technical expertise` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `build technical expertise` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `build technical expertise` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Public agencies must build technical expertise before they regulate new technology. 译：公共机构在监管新技术之前必须建立技术专业能力。&lt;br&gt;2. Public institutions should consider how build technical expertise affects fairness, efficiency and trust. 译：公共机构应考虑 build technical expertise 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss build technical expertise without ignoring long-term responsibility. 译：一个成熟社会可以讨论 build technical expertise，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：学习教育、职场发展、科技治理。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：expertise
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：专业知识；专门能力。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：不可数名词，常搭配 technical/legal/scientific expertise。 例：The expression `build technical expertise` should be interpreted through its context. 译：表达 `build technical expertise` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：build technical expertise；本卡覆盖这些变体：expertise
-&lt;b&gt;作文应用&lt;/b&gt;：可用于科技创新/科技伦理作文。可写：`Technological progress should be guided by clear rules and social responsibility.` 译：技术进步应当由明确规则和社会责任来引导。 适配话题：科技生活、社会责任、道德文明。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：专业知识；专门能力。例：Public agencies must build technical expertise before they regulate new technology. 译：公共机构在监管新技术之前必须建立技术专业能力。 2. 文章义/考试义：不可数名词，常搭配 technical/legal/scientific expertise。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Public agencies must build technical expertise before they regulate new technology. 译：公共机构在监管新技术之前必须建立技术专业能力。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how build technical expertise affects fairness, efficiency and trust. 译：公共机构应考虑 build technical expertise 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1365,7 +1329,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：监督 与 被监督对象/被监管
 &lt;b&gt;考研核心考点&lt;/b&gt;：同根词对比：oversee/oversight/overseen
-&lt;b&gt;词汇拆解&lt;/b&gt;：oversee = 监督；oversight = 监督；overseen = oversee 的过去分词｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：regulatory + oversight。中文：regulatory 表示“监管的”，oversight 在这里是“监督/监管”，不是“疏忽”。English: `regulatory oversight` means official supervision of an industry or organisation.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：oversight 也可指“疏忽”，但监管语境多为“监督”。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、制度语体。</t>
         </is>
@@ -1377,14 +1341,13 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能考 oversight 的两义。
 &lt;b&gt;答题技巧&lt;/b&gt;：看搭配：regulatory oversight = 监管；an oversight = 疏忽。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：supervision; monitoring; scrutiny; regulated entities
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulatory oversight should be strong enough to protect the public but flexible enough to allow innovation. 译：监管监督应当强到足以保护公众，同时又要灵活到能够允许创新。&lt;br&gt;2. In an exam passage, `regulatory oversight` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`regulatory oversight` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `regulatory oversight` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `regulatory oversight` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Regulatory oversight should be strong enough to protect the public but flexible enough to allow innovation. 译：监管监督应当强到足以保护公众，同时又要灵活到能够允许创新。&lt;br&gt;2. Clear public rules can make regulatory oversight safer and more accountable. 译：清晰的公共规则可以让 regulatory oversight 更安全、更可问责。&lt;br&gt;3. Without social responsibility, regulatory oversight may create risks that spread beyond one company. 译：如果缺乏社会责任，regulatory oversight 可能制造超出单个公司的风险。
 &lt;b&gt;其他可用地方&lt;/b&gt;：公共治理、职场管理、社会责任。
 &lt;b&gt;归一化合并&lt;/b&gt;：本卡覆盖这些变体：oversight &amp; overseen
 &lt;b&gt;归一化合并&lt;/b&gt;：原表达 `oversight of the overseen` 已改为考研一可迁移原型 `regulatory oversight`。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：监督 与 被监督对象/被监管。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：oversight 也可指“疏忽”，但监管语境多为“监督”。 例：The expression `regulatory oversight` should be interpreted through its context. 译：表达 `regulatory oversight` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：regulatory oversight；本卡覆盖这些变体：oversight &amp; overseen
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：监督 与 被监督对象/被监管。例：Regulatory oversight should be strong enough to protect the public but flexible enough to allow innovation. 译：监管监督应当强到足以保护公众，同时又要灵活到能够允许创新。 2. 文章义/考试义：oversight 也可指“疏忽”，但监管语境多为“监督”。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Regulatory oversight should be strong enough to protect the public but flexible enough to allow innovation. 译：监管监督应当强到足以保护公众，同时又要灵活到能够允许创新。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：科技创新、科技伦理、社会责任。套用句：Clear public rules can make regulatory oversight safer and more accountable. 译：清晰的公共规则可以让 regulatory oversight 更安全、更可问责。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1403,7 +1366,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：巨大的主权权力
 &lt;b&gt;考研核心考点&lt;/b&gt;：政治经济类立场词
-&lt;b&gt;词汇拆解&lt;/b&gt;：immense = 巨大的；sovereign = 主权的/至高的；power = 权力/强权｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：immense + sovereign + power。中文：sovereign = 主权的/最高的，power 在政治语境中是权力而非能力。English: `sovereign power` means the authority held by a state.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：power 在政治语境中不是电力/能力，而是权力、政权或强制力。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、强政治色彩。</t>
         </is>
@@ -1415,12 +1378,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：推理题会考是正当治理还是霸权/过度干预。
 &lt;b&gt;答题技巧&lt;/b&gt;：看到 sovereign，联想到国家主权、独立、最高权威。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：vast state power; sovereign authority; supreme governmental power
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Immense sovereign power should be used with caution and public accountability. 译：巨大的主权权力应当在谨慎和公共问责下使用。&lt;br&gt;2. In an exam passage, `immense sovereign power` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`immense sovereign power` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `immense sovereign power` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `immense sovereign power` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Immense sovereign power should be used with caution and public accountability. 译：巨大的主权权力应当在谨慎和公共问责下使用。&lt;br&gt;2. Public institutions should consider how immense sovereign power affects fairness, efficiency and trust. 译：公共机构应考虑 immense sovereign power 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss immense sovereign power without ignoring long-term responsibility. 译：一个成熟社会可以讨论 immense sovereign power，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：国际关系、政府监管、公共权力边界。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：巨大的主权权力。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：power 在政治语境中不是电力/能力，而是权力、政权或强制力。 例：The expression `immense sovereign power` should be interpreted through its context. 译：表达 `immense sovereign power` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：immense sovereign power
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：巨大的主权权力。例：Immense sovereign power should be used with caution and public accountability. 译：巨大的主权权力应当在谨慎和公共问责下使用。 2. 文章义/考试义：power 在政治语境中不是电力/能力，而是权力、政权或强制力。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Immense sovereign power should be used with caution and public accountability. 译：巨大的主权权力应当在谨慎和公共问责下使用。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how immense sovereign power affects fairness, efficiency and trust. 译：公共机构应考虑 immense sovereign power 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1439,7 +1401,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：战略利益
 &lt;b&gt;考研核心考点&lt;/b&gt;：国际关系/经济类高频名词短语
-&lt;b&gt;词汇拆解&lt;/b&gt;：strategic = 战略性的；interest = 利益/关切，不是兴趣｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：strategic + interest。中文：interest 在国家/政策语境中是“利益/关切”，不是“兴趣”。English: `strategic interest` means a long-term national or institutional concern.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：interest 在政治经济中常译“利益”，复数 interests 更明显。
 &lt;b&gt;语气色彩&lt;/b&gt;：正式、国家政策语体。</t>
         </is>
@@ -1451,12 +1413,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：选项中 national security concern/economic benefit 可能替换。
 &lt;b&gt;答题技巧&lt;/b&gt;：interest 若在国家/政府语境，优先译“利益”。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：national interest; strategic concern; long-term security interest
-&lt;b&gt;多场景例句&lt;/b&gt;：1. A country's strategic interest may shape its policy on advanced technology. 译：一个国家的战略利益可能会塑造其先进技术政策。&lt;br&gt;2. In an exam passage, `strategic interest` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`strategic interest` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `strategic interest` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `strategic interest` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. A country's strategic interest may shape its policy on advanced technology. 译：一个国家的战略利益可能会塑造其先进技术政策。&lt;br&gt;2. Public institutions should consider how strategic interest affects fairness, efficiency and trust. 译：公共机构应考虑 strategic interest 如何影响公平、效率和信任。&lt;br&gt;3. A mature society can discuss strategic interest without ignoring long-term responsibility. 译：一个成熟社会可以讨论 strategic interest，同时不忽视长期责任。
 &lt;b&gt;其他可用地方&lt;/b&gt;：国际关系、科技强国、经济安全。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：战略利益。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：interest 在政治经济中常译“利益”，复数 interests 更明显。 例：The expression `strategic interest` should be interpreted through its context. 译：表达 `strategic interest` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：strategic interest
-&lt;b&gt;作文应用&lt;/b&gt;：可用于考研英语一作文中的“原因-影响-建议”结构。可写：`This issue shows that public interest and long-term development should be given more attention.` 译：这个问题说明，公共利益和长期发展应当受到更多重视。 适配话题：社会责任、科技发展、教育学习、职场发展。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：战略利益。例：A country's strategic interest may shape its policy on advanced technology. 译：一个国家的战略利益可能会塑造其先进技术政策。 2. 文章义/考试义：interest 在政治经济中常译“利益”，复数 interests 更明显。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：A country's strategic interest may shape its policy on advanced technology. 译：一个国家的战略利益可能会塑造其先进技术政策。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：文化交流、社会责任、个人品质。套用句：Public institutions should consider how strategic interest affects fairness, efficiency and trust. 译：公共机构应考虑 strategic interest 如何影响公平、效率和信任。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1475,7 +1436,7 @@
         <is>
           <t>&lt;b&gt;字面含义&lt;/b&gt;：无差别关税；不加区分的关税
 &lt;b&gt;考研核心考点&lt;/b&gt;：经济政策负面搭配
-&lt;b&gt;词汇拆解&lt;/b&gt;：in- 否定；discriminate = 区分；tariffs = 关税｜中文：把这个表达当作一个整体词组来背，重点看核心词、介词和搭配对象。 English: learn it as a reusable chunk; notice the head word, the preposition, and the noun it commonly takes.
+&lt;b&gt;词汇拆解&lt;/b&gt;：indiscriminate + tariffs。中文：in- 否定，discriminate = 区分，tariffs = 关税；整体指不加区分的关税。English: `indiscriminate tariffs` are broad tariffs imposed without careful distinction.
 &lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：discriminate 既可指区分，也可指歧视；indiscriminate = 不加选择的。
 &lt;b&gt;语气色彩&lt;/b&gt;：批评性，暗示粗暴和低效。</t>
         </is>
@@ -1487,12 +1448,11 @@
 &lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 negative 信号明显。
 &lt;b&gt;答题技巧&lt;/b&gt;：impose indiscriminate tariffs = 无差别加征关税。
 &lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：blanket tariffs; across-the-board tariffs; arbitrary duties
-&lt;b&gt;多场景例句&lt;/b&gt;：1. Indiscriminate tariffs can hurt consumers without solving deeper economic problems. 译：无差别关税可能伤害消费者，却无法解决更深层的经济问题。&lt;br&gt;2. In an exam passage, `indiscriminate tariffs` may signal the writer's attitude, a cause, or a contrast. 译：在考试文章中，`indiscriminate tariffs` 可能提示作者态度、原因或对比。&lt;br&gt;3. When writing about social change, students can use `indiscriminate tariffs` to make the argument more precise. 译：在写社会变化类作文时，学生可以使用 `indiscriminate tariffs` 让论证更精确。
+&lt;b&gt;多场景例句&lt;/b&gt;：1. Indiscriminate tariffs can hurt consumers without solving deeper economic problems. 译：无差别关税可能伤害消费者，却无法解决更深层的经济问题。&lt;br&gt;2. A government that imposes indiscriminate tariffs may protect a few firms while raising costs for many families. 译：一个加征无差别关税的政府可能保护少数企业，却提高许多家庭的生活成本。&lt;br&gt;3. Trade policy should avoid indiscriminate tariffs and target the real source of unfair competition. 译：贸易政策应避免无差别关税，并瞄准不公平竞争的真正来源。
 &lt;b&gt;其他可用地方&lt;/b&gt;：经济生活、国际贸易、政策批判。
-&lt;b&gt;考研英语一适配&lt;/b&gt;：本卡保留是因为可训练科技政策类阅读、态度推理、熟词僻义、完形搭配、篇章逻辑或作文迁移；过窄技术项已剔除。
-&lt;b&gt;多义项详解&lt;/b&gt;：核心义：无差别关税；不加区分的关税。 语境义：在本文中按文章主题理解，重点服务阅读定位和翻译。 拓展义：discriminate 既可指区分，也可指歧视；indiscriminate = 不加选择的。 例：The expression `indiscriminate tariffs` should be interpreted through its context. 译：表达 `indiscriminate tariffs` 应通过语境来理解。
-&lt;b&gt;原文/拓展表达&lt;/b&gt;：indiscriminate tariffs
-&lt;b&gt;作文应用&lt;/b&gt;：可用于经济发展/就业创业作文。可写：`A healthy economy depends on both innovation and prudent regulation.` 译：健康的经济既依赖创新，也依赖审慎监管。 适配话题：经济、职场发展、社会责任。</t>
+&lt;b&gt;多义项详解&lt;/b&gt;：1. 核心义：无差别关税；不加区分的关税。例：Indiscriminate tariffs can hurt consumers without solving deeper economic problems. 译：无差别关税可能伤害消费者，却无法解决更深层的经济问题。 2. 文章义/考试义：discriminate 既可指区分，也可指歧视；indiscriminate = 不加选择的。 3. 做题提醒：如果选项只保留字面义、忽略搭配对象或语境色彩，通常是干扰项。
+&lt;b&gt;原文/拓展表达&lt;/b&gt;：Indiscriminate tariffs can hurt consumers without solving deeper economic problems. 译：无差别关税可能伤害消费者，却无法解决更深层的经济问题。
+&lt;b&gt;作文应用&lt;/b&gt;：适配话题：经济发展、公共政策、社会责任。套用句：A government that imposes indiscriminate tariffs may protect a few firms while raising costs for many families. 译：一个加征无差别关税的政府可能保护少数企业，却提高许多家庭的生活成本。 改写提示：保留目标表达的核心搭配，根据作文主题替换主语、宾语或评价对象。</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">

</xml_diff>